<commit_message>
Update inventory — 03/08/2026, 9:45:42 am
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,16 +417,33 @@
         <v>Created</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>New box</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-08-02</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,9 +459,23 @@
         <v>Notes</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>power Adapter 12v / 3 amp</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory — 03/08/2026, 11:25:31 am
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -422,10 +422,10 @@
         <v>B001</v>
       </c>
       <c r="B2" t="str">
-        <v>New box</v>
+        <v xml:space="preserve">Test 1 </v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Top shelf in storage room</v>
       </c>
       <c r="D2" t="str">
         <v/>

</xml_diff>

<commit_message>
Update inventory — 3/8/2026, 5:33:19 pm
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -443,7 +443,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -464,18 +464,46 @@
         <v>B001</v>
       </c>
       <c r="B2" t="str">
-        <v>power Adapter 12v / 3 amp</v>
-      </c>
-      <c r="C2">
+        <v>HDMI cables</v>
+      </c>
+      <c r="C2" t="str">
+        <v>51</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B3" t="str">
+        <v xml:space="preserve">IEC POWER CABLES </v>
+      </c>
+      <c r="C3" t="str">
+        <v>15</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4">
         <v>1</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory — 3/8/2026, 5:34:21 pm
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,16 +434,33 @@
         <v>2026-08-02</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>B002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>New box</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-08-03</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -501,9 +518,37 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>B002</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>B002</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory — 3/8/2026, 7:56:30 pm
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,48 +419,31 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>B001</v>
+        <v>box01</v>
       </c>
       <c r="B2" t="str">
-        <v xml:space="preserve">Test 1 </v>
+        <v>New box</v>
       </c>
       <c r="C2" t="str">
-        <v>Top shelf in storage room</v>
+        <v/>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>2026-08-02</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>B002</v>
-      </c>
-      <c r="B3" t="str">
-        <v>New box</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
         <v>2026-08-03</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -478,13 +461,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>B001</v>
+        <v>box01</v>
       </c>
       <c r="B2" t="str">
-        <v>HDMI cables</v>
+        <v>IEC power cable</v>
       </c>
       <c r="C2" t="str">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -492,13 +475,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>B001</v>
+        <v>box01</v>
       </c>
       <c r="B3" t="str">
-        <v xml:space="preserve">IEC POWER CABLES </v>
+        <v>HDMI cables</v>
       </c>
       <c r="C3" t="str">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -506,7 +489,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>B001</v>
+        <v>box01</v>
       </c>
       <c r="B4" t="str">
         <v/>
@@ -515,40 +498,12 @@
         <v>1</v>
       </c>
       <c r="D4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>B002</v>
-      </c>
-      <c r="B5" t="str">
-        <v/>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>B002</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Y</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory — 3/8/2026, 7:57:29 pm
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,16 +434,33 @@
         <v>2026-08-03</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>box02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>New box</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-08-03</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -501,9 +518,37 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>box02</v>
+      </c>
+      <c r="B5" t="str">
+        <v xml:space="preserve">1060ti </v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>box02</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2060ti</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory — 04/08/2026, 7:19:54 am
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,6 +416,9 @@
       <c r="E1" t="str">
         <v>Created</v>
       </c>
+      <c r="F1" t="str">
+        <v>Photo</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -433,6 +436,9 @@
       <c r="E2" t="str">
         <v>2026-08-03</v>
       </c>
+      <c r="F2" t="str">
+        <v>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/4gHYSUNDX1BST0ZJTEUAAQEAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADb/2wBDAAoHBwgHBgoICAgLCgoLDhgQDg0NDh0VFhEYIx8lJCIfIiEmKzcvJik0KSEiMEExNDk7Pj4+JS5ESUM8SDc9Pjv/2wBDAQoLCw4NDhwQEBw7KCIoOzs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozv/wAARCAF3AfQDASIAAhEBAxEB/8QAHAAAAgIDAQEAAAAAAAAAAAAAAAECAwQFBwYI/8QAUxAAAQMCAgUGBwsJBgUEAwAAAQACAwQRBSEGEjFBURNhcYGR0QciUlShwfAUFhcyU1WSk6Kx4RUjM0JDREVjgzVicnOCoyQlNNLiZISUwqSy8f/EABoBAQEBAQEBAQAAAAAAAAAAAAABAgMEBQb/xAAmEQEAAgEEAgIDAQEBAQAAAAAAAQIRAxITMQQhFFEiMkFhBUKB/9oADAMBAAIRAxEAPwD1haNYElMpH1qS/NPpI2CVgVKye9BEAIsE0IEQjVFk0Khao2ILQmhBHVCLDbZNCBWTAQkgLDelbgLppKgsBzEcUAWzR0A5IOfFAWF89/Ynluub5bc0iTvFudHbxzCIMri5358yGgNO+wz22si5ve23Pbkjq9KB6oN7dpICPFGTr7EA57r223Rewt6UDs3Kw7c0ZjLLI5Z70gee6Bfbs6QiF4t/i3tzbPQm0eSCehFjsIJPOjLe6x32zQMAEi9jwuUrNJ2bdvEp34jdlxSu7abdKoRAGW9FrA7OxMWDhsPMgEm4I699lQiPFsdnC21GrkQBkO2yNYtO/PNAB29mSAI32uiwtsAQi/EAooAvsyT3XG9K/MLpoAgbLIIyQjqQLehBzQgE0k0AlZNJAW5kWQhAW6EWbwTJQDuVQWvtStY8UztvxSvnfNFMNtcbPX7XRqttmL79qMzzX9ro5gLqofi5HbY5jilqtzG4JnMbALozFs8r9aoRA1bC3EJhtrnxb7jvRtabCynrPubAHcbjYUgBIsA5otrXz9KQaB4xuC3cDZIWLsibeTe9ky0EnVPi7s1Q7AHYAbZpWaWgEtDto5kr5jVeSU2nK1za+ZKZQODgfFcWjhdCkDrZl4H+J1vUhX0K3fFKkk4ZFA2LzNhNCSAQhCAR1oQqBBQkgEIRZAkJpIBJCFQ8rdCVs+KYF8uKSAujj6UXuANlkXy2nPaOKINhG870gL9CY4bkr2tvVDsBfbzIPEX2I2ZJAAgiyB2y9tqedja+e07VEHPcn07uZEAIG0cyeRve3WkObZfJLabceZAza+7qQTfK/TlZHMf/AOpXtvNt6BngTYHpRkQN557qJ6kHoFuCoOfLqT2brZJW3HbfsT3Dh0oADaPQjbwSG1PcEUxkhGYPBLtQNCSEDQkmgEIQgDtRfNCEAhCEAmD0pIVD27ckC1yL7SlY2zQgYzzJtZF7hG7JA2WyVQwXGwtlsQTexyy2JXvmSSd90yLm3P0ZoHfmJyvmEtpF+G8pGwGVwmAA7LdzKiWdwbgDddIiwtY3323XUQDfIjiLm10zttnt3FVDvck26bZIPjA2vnxQNhte2642oBBsANp3DMqKlrMZkWNdz6pQlc/qkt4gcUKgSGxNILztGhCEAhCFQJbNyeaRQCW5BQgEISugaWaEkDRwHYkhUOxI2FLPZdFkelAcyXrRmEA250QFF89pQhUHVZHPvCPQkMige7m3I3bfSlu3J57EAb32Ivlnmltz9SPvQFwRmjZlstxzslnnvRf23oHfKwKLi+ZUev8ABF7EKiVxxCD2JXPoRsRD2o9tqE1AbkIR7bVQAoRdCKaSEIBNJNAIRdCAQhCASTGxF1QZ238EZ70IuqA7b8UwSDcXBS28yOfeUQHp7U8srZbkHK6V78boHsIzsUbwbXuOtF87WHajPs3Kh7MjccbFDbHIm18kjYZ52tndG8gEX4IH1m6Dq5ndfednSle1skwdU7L7rIES3e25G9CbSQMnDsQglcAEk2AC1xx3CWEk4lTW3DXCzZBrRuHEZrjVbGYKyaI/qSOHYU0dKNTOUvba6udIsFH8Tp/ppHSXBB/E4PpLkN0wV6PjV+3Pll1z30YHfPEoO0qJ0pwMfxKH09y5OhPjV+zll1b314F84xnoae5I6XYCD/aDfoO7lyq6RV+NU5JdU992AD9//wBt3conTDAfPj9U/uXLErp8apyS6idNMCAyq3E/5T+5I6aYFb/qZCf8p3cuXphPjUOSXTTptgY/bSnoiKj798E+Um+rXNbpJ8ahyS6WdOMF3OnP9P8AFI6c4MPOPqx3rmqLq/HonJZ0g6d4R5FSQf7g71E6e4OP2dV9Ad651miyfHoclnRTp9hG6Gq+g3vUTp/hI/YVX0W9652kr8ehyS6H8IGFHZT1X0W96PhAwvzap7G9650SAi+afHockuiHwgYZupansb3o+EDDh+61H2e9c7Urq/Hockug+/8Aw+3/AElR9nvT9/8Ah3mtT9nvXPboup8ehyS6F7/8O81qfs96Pf8A4b5rU/Z71z3WRdX49DfLoJ0/w3zWp7G96R8IOG7qSq7G9659dRJT49E5JdB+ELDfNarsb3pjwh4Z5pVdje9c8ui6vx6HJZ0P4Q8N80quxven8IeGeaVPY3vXO7ounx6HJLog8IWG+aVP2e9P4QcO81qfs9650mnx6G+zovwg4b5rU/Z70vhCw63/AElT9nvXO0XV+PQ3y6H8IWHeZ1P2e9MeELDvNKntb3rnJcgOuU+PQ5JdHHhAw/zSo7W96fwgYdfOlqLf6e9c7undPj0OSXQ/f/h3mtR9nvTGn+HH91qfs9654DmpAp8ehyWdB9/uHea1PY3vUvf7hvm1T2N71z29kEp8ehyWdDGnmF/IVX0W96Y07wo/sar6Le9c8BTur8ahyWdDGnOEnbHVfQHepDTjCPIqvqx3rnYKYKfHockuiDTfBz+rUj+mO9SGmmDnzgf0x3rnV00+PQ5JdH9+OEH9acf0/wAUe/HBvlZvqlzoEoyT49Dkl0b334Lf9NKP6RT99+C+cSfVuXOFHWU+NReSXSvfdgpP/Uv+qcn768F86eP6bu5c1BKd8r36k+NU5JdXocTo8SY91JNygjIDrtIsTs2rKyJ2ALzOgkdsMnlP601uoAd69P0/evHqVitsQ61nMA7Eb+CezpSGef3rCg557UJi+6/UUKgIuCFyXSWHkNIKxlsuUuOsA+tdcXNNO4OTx/lALcpG0/eFrxp/LDOp00uF4XLilVyMbg1ozc4i9gvRVOgc7cJGI0NR7oYRfVsLkc1lqNH8QjoKtwmyjlGqXcF6iXHIcIp9emqGMgF9WzruIz29q9N5vuiIcoiJh4QiySGyOmL5SLB7iQOZNdpYRSJTSKBJIQqBNRTQO6LpIVDQEkIZSukXKKLoZSukldB5jdB6jANHaCTD2Ylipc6KR3iMa6xte2xWaT6K0NHRyYjhE2vTxODXtJ2X9tipwTH6FuEtw+teIponExSOGVjnkdxWNjmkDKikdQ00weJXDWaz4oAN7nnXGsX3+2/WGh2IugqN13YSLkaygSldMCzWSLlC6LpgSLkrqN0XVwiV0XUboumBK6AVG6YKuBIKSgCpJhTCHZBCCLhVHrsG0Yw0YO2vxV7i6QBzIwdoJ3Dm2lYGlOjkGDspK2inbLSVYOrY31SN11dh2lcMVBBT1DjFLDGYiS24c3ZcZHOy12OYx+VHxxxlxgivqlwtc8w3BcNOL7p3NTjDVgp3UdiLruzlO6YdZQTuqZTundQundDKd0wVAFMFBMFSUAVJBIFNRumFFSuU1FSagYC22jOCw41XPE8wip4ra7t1zsC1jWgqWFV82ETyxSxSOilcDrMBNj1LF8zX8SO3qa/RzDpsNqZqImOWmFyLEAjZnfevHjavQ4hjkb6d0dMCXyiz3lpH35rQBuaUice1l0TQ2PU0eYcvGe53pt6lv8uZarRmPk9HqP8AvM1u03W16sl83UnNpeivRXz4oAPDNCe1YU9Vx2AlCWqOHoQgkvB+EOH/AIilm4tLfSO9e8XkPCBFehppLbHkdo/BNGcXhL/q5+gNadrR2KSF9J5jtkkQdwv1J3Up3uGB1wa9zc4j4ptca1j96sRmcCuzuB7CkWngexYNES+C7iSb7yr9VWYxOBcWngexLVJ3FUlqWqmBfqO4Jhh4ekLH1EtQcB2K4Msrknc3aEuTcOHaFjag4BGoOA7FcGV5Y7gO0I1TzdoVGoOA7EanMEwi6x5u0ItzjtCq1BwCWqOCu2BbmNjh2oseI7QqtQcEiwcE2i7UuLHVPWExHq7A0dBCxiwcAoFg4K7Rllp5u0KJa7gO0LE5MKBYOCu0yzdR3AdoS5OTyftBYOoOAUSwcFdqZbDkpPJ+0E+Rl8n7Q71rdQcEaiu0y2XIy+T9od6ORk8n7Q71reTCfJAptMthyUnk/aHejk3+T6QtcY0uTTaZbLkn8PSE+Tf5PpHetbyfMpiMcE2JlsBG/wAkdoUtR3D0hYIYOA7FNrBwHYm0yzNR3D0hGo697DtCxg0cPQnYcAphcsmxtu7Qkedze1Y9glqq7Uyvs35Rn0kWb8rH9JUanMjV5kwZZFm/Kx/ST8X5WP6Sxw2+5PVVwZX+J8qztQHM+UZ2qjVRqpgyyQ5nyrO1MFnyrO1YwCkGqYXLJuz5ZnanrMB/Ss7VQGjgpBt+CmFXa0fyrO1SBZ8oztVIaFLUCC3WZ8qztTD4xkZo7/4lTqjgtXiX6YDg1Igy9CWvjtcbQCOhTbOQ2ylXHk6kxtyDGtb2ABYussQq15vmoXtnzXUdZNo13BnlHV7UkdYwqHkMJpIsvEgYPQFljnzUYxqxtblkLKS+Tbt6o6GSEdqFlRbmQn0WQga85pxFr4AX2/RyNPq9a9GtVpNDy+j1Y3baPW7M/Us0nFoLdOTpJnaUl9V5Aro2iSgxCMi96ZzgP8JB9SousrDfGqnR/KwyM7WFajsaTDnXjeOdZq1+HHxnhZ63fsjokIQshFCElYhDQhex8HOHUGJ4lVRV1LHOBEHNDxexuulK7pwzM4eOsiy7qdE8AH8JpvoJe9XAPmml+rC7cP8ArHI4WhdyOiuA/NNJ9WEjotgOz8k0v1YTh/1ORw09CRXcTotgPzVS/VhROi2A/NVL9WFeH/V5HDiSoOK7idFcB+aqX6CrOiuBfNdN9BXhORw+6g4ruJ0UwHfhdP8ARUTopgHzXT/RV4U5HDr2UbruDtEtH/mqD6JVbtEtH/muDsKvFJvcTui9l2o6J6P7fyZB2HvUfeno+P4XB6e9OKTe4ttKkF2f3p6P2t+S4Owp+9TR+/8AZcHYU4je4uhdqGiuAfNcHYpDRXAPmun+inEm9xQKY612waLYB810/wBBTGi2AfNVL9AJxG9xIA86mAeC7a3RfAPmmk+qCtbozgI/hNJ9SFOI3uHgHgnnwK7mNHMD+aaP6lvcpjR7BPmmj+ob3JxHI4TY8D2JXttyXe24Fg42YZSD+g3uVjcGwsbMPph0RN7leJOR8/GZg2yNH+oIE7PlGfSC+hRhmHt2UdOP6Y7lYKCkGylhHQwJxnI+eBNGD+lZ9IJiRh2Paf8AUF9FNpKcbIIx/oCkIIRsiZ9EJxnI+dQL7BfoUuTfuY49S+ixDF8m3sTEUdviN7E44OR85kFpzBHSEA2Xq/CS4HSt7WgANiYMuteTXK1cTh0rOYysBUgq27VYFzluEwpKAUgsqa1k7OXxOOLbrPa3tK2awKNnLaQ07f5zfQfwWoSW6xBwNdMRs1ysZTqH6873cXEqsFYiPTSV1k4azlcTpY9utM0ekLFK2ejcfK6Q0TbXtLfsF/Upb1WSO3VSjnvZMDJC+Q9QQiyLZKKLc5QixQgax6+PlaCeM/rRuHoWQovzaQucdrLirxZxCgsmvjbDWTR53bI9pHQSFjFfXj3DyT2Svw9+piNOf5jQegmx+9Y5TifqTMf5LgVqBrKccnXSx8CR2FZyxq0CLH6po2cs+3aVfrLpftmElElInNF1hTuldK6LrUIkF7PwYS6ukkjNz4HfeF4u69T4OpeT0tgHlse30Ltp/sxbp2VyipHYokr1uCJUTdMu51AniqgJUCbBDnKsuQNx4lVudYIc7JUverAk5ygX86rdLzqp0nOqLi9QMmeaoMnBQMmSqr9eyXKcVjGXikZBxUGTyme1PlFicpzpiS29BliTnUg9YYk51NsiIzGvzyKsa9YQkVjZEGa16mHLEa/LarGvzTCMoOyUg5UNdzqYcoLgc1MOVIcpgoi0FSuqwVIFRFgUgqwc1MFFTT3KIKZPinoQcU8IL9fS2q/u6o9AXmwt7prJymldcb3tJb0BaILhqfs706SCsCgFNcZdYSCkoBSWVBOSxMHGvj8bvJc53YCVkuNgVj4E0uxKZ9/iQyO9XrT+Sk9sxx8bNAKTjmelK6ipXW+0Mj5TSSE+Qx7vRb1rz+1eq8H8WvjE8nycGWXEhc9WcUlqv7OhppBNfJeoIskmgEIQgEEW3oSXJXJtJouR0grWWy5UkdYB9a1K9Jp1CYtIHPtlJG13q9S80V9bTnNIeW3YKSEl1RRjIAx57gLB7WOHWxp7073CnjxPK0M+Xj0rBfnBIKqB8ULpPUM/0yUrpEpXWcKlfNF1G6LrSJ3W90Jl5LS6gN7XkLe0Fefutjo/PyGkFBLs1ahnpNvWulO4Yt0+gL+KoFyWtdoUC5ex55MlQLski5VuciG52Src7NRc9Uvk25qiTn2zKofJzqL5M9qodJzqqm9/OqXSc6rfIqXSZoq4yc91AyLHdLbeqzKgyTIomQLFMqiZedRWWZQjleKw+VtvRyt0RnCUKYk51gCXnUxKhhsGyKwSc6wGy86tbIiNg2S6ta/isBsmxXNkRGe16ta66wmPVzXoMoOVgcsZr1aCiLw5WArHDlYHKIuBUwVUCpgoLApHYqwVJ5swlIHBtJ36+klc7jM771rAVk4xKJcYq3g3Bmd95WKFwv29NekwpjYqxZTC4y3CQKd1EFO6y0Uhsx3QoaPs/wCumv8AFhDe1w7kpzaF/QrcDGrhldJ5TmM+8pP6p/TJzRfNQJRdQTuvceDqPKulI8hoPavDLofg8j1cKqJPKm29AHeuHkTikumn+z1qe5JPrXzHpCEIQNCEIEkmkuSvBeEOK1ZTS2+Mwt7D+K8YV0Dwhw61DSzD9WQtPWL+pc/K+n485pDzX/Ykr2SKRXoYRxm78NoJL/EMjD9K49BWOx12NPMsjEAHYI1182VJFuYs/wDFYkRvE08y6f8AlP6sJySuglRugd0XSORSJVRLWzV9FJyVbDIT8SRruw3WMFJhs7pXSvbMvomN+tC13EKLnLHw6blcNp5L31omn0Kxzl7HmNzlU5/OoucqnOVQ3vVD3oe9Y0j1VDpFQ+TnSe9Y73qKm6TqVDpOdQe9UPkUVY6RQdJ2Kh0nOqnSIrIdLzqszc6xjJzqBkUXDK5dMTZ7VhGVLlUyNiJudWNm4la4Sq1siZGxbIrmSLXMkWQyTnUymGwZJszV7JFrmPWSx90RnsfeyvY9YMblkRv2K5RmsddXtcsKNyyGOVRkhymHKhrlY0qMr2uVjXLHaVY0oLgUTv1Kd7uDSfQotKoxWTksJqpL/FhcfQVY7Hz/AFD9eokff4ziVFpVZKYK81npr0uBU2lVAqQK5y0sui996jdFwstq6l35h3QsnDPEwSQ75J/ub+Kwqo/mDzrNphqYJT5/Ge93pA9Sk9J/UCUrpXQoJ3XT9BY9TRmN+zlJHnsNvUuXA5rr2isPIaMUDd5hDz0nM/evN5U/hh10u23CaQTXznoCEIQCEbEIEjYEJLmrz2m8PK6OyOtnE9rh229a5eV17SOHl9H6xn8onszXInCxXv8AFn8ZcNTtAqJUioletyTnYJMDqxa5jkjeO0j1rW0xvF0LbQeNQ4hF5VMSOlrge9aikP5vrXSP1Z/q4pb0ykUVFxzyUSUztUSVqGZO6A7NRulddIZl3jRubldHKB4zvA37lnOctFoTNyuiVDnsYW9hIW6eeK9kPPKD3c6pc5TcbA8ypebKsq3uWM929WyOWNI5GoVvesd71N7ljSOzUVF71jyP2qT3WWPI7NRQ+RUuk50nvVL3qS1CTpFWZRfaqnyZ5FUOlzWJlrDJM1kuWusMyc6BJmplWwbLe2avbJzrWNkKyI5edMphsmSLIjfzrXRvyWVG9ahlsGOWRG7NYMbrrJjcqks5judZDHLCjdkshjkRmsfuWQxyw2FZDHKsyy2lWAqhhurWlEXNKsBVTSptKrK5pWu0nk5LRrEX3tanf9y2DStLppLyeiVfntjt2kKwOHOPjHpSBUSc0ArzS9MLgVK6qBUg4LnLa3WQSoXQSsSqqrd+btzrY21MIom/yy49biVqqo+IOlbisBjgpI97KeO459VSf4QxE7qN07qKla4sNp2Lt1BEIcPpogLBkTR6AuK0kfK1cMflyNb2my7g0WaBlkF4vLnqHbSSuhMI3Lwu46kIQgaEWQqIpIQuaqK2ITUU8R/XYR2hcWkuHZix3jgu3OF2kcVxrFoTT4pVREW1JXDozXs8We4cdRhFIppHYvc4r6Lxpnxk5SRSM+yVpqQ/GC3OHkDEIOBeAevL1rTRAx1UkZFiCQR0LpXqWZZF7KKnvUSMroqDsiolMqJW4ZlEpXTKiVqEl1TQjFGUeiELpGueBM9ni2yzJW8OPQEZQyeheK0Sfr6J1DfkqwHtaFtA4AbuwL2V6cJj235xiF17MfzXIUDiLHfqHtWna4WUw/K9htyVymGxdWNJ2elVPmB4dqw9fLZ7e3txevl8Ue3t9/HOZkwucbg2sOtUPYTvA6/b260a+eX3qsu5z2+3t6JlUHRF21zRn7e342qdTOP64CsLyXbd/t7ewjr5/G5tv4JlVDqIk/pBboVTqB1v0o2cPb29OW943ut7dCg523O+XeoMJ+Fk/th9H29uq9TsJJ/b/YK2Jcbdqhc2KzhrMtccI2/8R9gpDCbEfn/srY3JJUCUwZYX5PDf232VIUgb+09CyXdCsFJLa7xyYOYLza/QPbvyvtjNGpbPcr4Jda4I2KqUshzDS4gfrbOxVUM75jIXG9iAOZInJhto3LKjcsGMrKjK2xLNjKyGFYkZWSw3KqMuMrJjKxGHNZMZVZZTCrmqhhVwKIubsVjdiraVYFUWNXnvCC7U0Qqzx1R6QvQtXl/CVJqaIyNv8aVgRIcZ3pgqJ2o3Lzy9MLAVJpJKlSUz6qQtYQ1rRrPe74rBxKyDNQQkiKmNRb9pM4tB6Gg/fdc5luGNdBKy2zUFQdSWn9yk5crE4uaOlp3dFljVUMlLO6GSxc3eNhG4jmWFYtRmQ0Z8FvMWI92uaNjAG9gC08TTJXU7AL3eBbrWzxB4fWyu4uP3qW/hHTGKSLpKK2ej8fLY/QxeVO30G/qXaAuR6Ew8vpVSfy9Z/Y09664Avn+VP5RD0aXRoRuTsvI6kmhCA6kIQgghCFhSO1cp0vh5HSOqG55D+0LqxXN/CBFqY0yS2UkQPYSvT404vhy1OnlEjdO4Rkdi+g4HE4slY/yXA+lYmIMMWPVQIsHSuI6Cbj0ELJcDYhRx235ZjmBymijf2tHculElQQokKwqOxBW4DioFWuCrK1CSrIUSrCoELcMvaaEu1sDxWPyXxye3YtwDlkPb2+7s0WgZ1ocVi4wB3YVu2nIZL10/WHGe1jTkPUmCbZ8OO326++sO8Ugp8o291pFl+nt9va/W78c1VygG8ZH29vYnK3I2HL29ujrgt1iTfM9agTmq+Vyztzmyi6Q3JyBt2IqROaRI23t1+3sFWXm+Xt7ersC93sVBY6wBv7e1vbcnEDmUCSeHQm1r32AG1QGtkoZnIC63lDotiVY1rzEWRuF9d2QssyHAqKGVzZXyVLmH4sWTL/4t+3cs1tF5xX2WmKxmZebhpZ6l4ZHEXuccgMyVsafR5znltRJqkbY4wHv69w6z+Pq6Gjp3wlrZGxADxomDVaek7T1lSqKQUgaAGxtPjWaNq7xozM4lwnyKxOIecdQChN2RMYSDquvrvvbich1BaGpkczWDjra23WzJ9a9XWkVDQ2M6j4xk52wDpXmaunjiu+aUFxPxhv6OKzPjX/rrXXrhp3Mmqnagad+ZNgBzrKgpBSRMtdwkz17WDujmU6yVlJHeaPVLheOmO1395/Nzb1j0M8tS+WWdxc8uA6BbZzBctm2cOm7LYMWVEseMLKjGxahmWRHkVlM2hY8YWSwKoyI9yyI9qx4wsmNVmWQ3JXNN1SxXMzRFzVaFU1WtVRY1eO8KLiNG4m+VUN+4r2LOC8P4V5LYRRx+VMT2BP5JDlBzQMig7U2i56rrzy9DOceSwWFrcvdEjnP5w02A+8rBus+BhrqAUrD+fhcXxsP7Rp+MBzgi9ucrAsQSCCCDYjeFyhs9a3Ss+uOvhuHSO+Pyb2f6Q82WPSUclW86tmRMzkld8Vg5+5SxCpZPM1sNxDC0MjB22G885Oak9iOFsMmNUoG51z1Z+pWzEmRxO0lGBs18WMl7CKF7vs29alJE593N2XWZ7ajpSi69HRaC4/X0jaiCkBZILsDnWLuhaGop5aWofBPG6OWN2q5jtoKzFonoer8G8Ifj08pF+TpzbmJcF00Ln/gyhs+vm5mNv2ldAAyXzfInOpL06cfiaEk153QIshCAHR6EI6kIIJXTQsKRXhvCPBlR1AHlMPoI9a9yvL+ECLXwFj/k5ge0EetddGcakMXj8XidGKOlrcZaysGtExpeWHevZVrMFrMKFOcObBICfzjbawNti53Tzy0lQ2eB5ZIw3BC2FXpBV1kHJPZG075GjxudfQtWZtEvPWWtBuXW2BxAPFVY0QWYdJb9jqH/AEuI+5WWAAAyCjizS7CaOQbGSSM//U96717ZlVuUSmzNgPMgqishRIVhCgVoVkKBCsKiVqGZen0Ad/zOsi+UpXjsW5a7xfxWg0EfqaTRt8uKRvoW+uAS3gvXp/q427TDm8T1I1h7H29vTFpado6c0tYXyA7VpE9ZGsoF2ez0o1uZQT1jb7kiczlkgZ3AVzYri5BIHMszaI7WIyx7knL0KwROd0ncthT0bpZTHEy+waxGzitrHhZkIjporxh3jzvOXP1XysuNtaInEOlaTLz7IHZZXXrMJw/DhTGanZLLK0C76mIhjegLNw/BsPbOXCMTubbMizR0Dvut4IwQGtFx0LMavv2mpWYjH9aeeeVzdV1TGBsNrgAdCwTqbGPLgObet5UYYwkvB37LKMeHB5ya7PbsX06eTo0j8YfJ+NqzbMyrwRjJg8PtrbnEbVh4zT1DZS+Yk0+9wO3mWwnhjoy0g2Bydbdzry2N6U8kTStLZYgcg4dy3XUzbkjpi2nbdsgVcEslm08IcCR4kcgJ681RjdVhWBUuqIm1Ne9viMc0ERZbT17FpWaTGnFQ+loKeGolyE7Bm0b7BefmkdI9z3uLnONyScyuGtq21Ix09+npRWcqppZJZHyyvc+R5u5zsyVsMHF45f8AGPuWscc1tcDF4Zf8Y+5cP67/AMbWNqyY2qtjFkxtWmZWxtushgzVTBxWQxqrOVsYWTGFSxuayGDYiLmK5oVbArmhEWNCsCg0KwBBNoXPfC0/8zh0f957vQF0NgzXNvC07/jMPZwjefSEnqVjtzghANjsUkrLzvQNhBblY5FZbcUrbDWkbJltkiY89rgSnT00EVKayrBcCbRQgkcpxJI3BS/LFYMoTFAzcyOFgA7QVzmc9NQonrKioaBNKXNGxuxo6AMljuzutlFyeKl0Too46vVJjdENUSkZ6pGy545LWuFiRvCkDYYDGXSV7wCXNp9UAc7gEM1qWojkmheGawJDmkEjftRg3i0GIyXtfUb6b+pVF7icyTbisT7mWo6dNh0g5SCKSCv5GOE3YdcfFXhdIK6PEsZnqo82uIGt5Vt61uvcW2DmQTdc6acU6amcukeDWLVwiqlP689h0Bo9ZK9kvNaARcnorC7fJLI4/SI9S9MF83WnOpL00/UIQhcmghCOpA0I7UIKkIQsKFpNMIuV0bqcs22d2FbtYONQmpwWsiG10LgOxapOLRKT043ZJSO2/HNIr67yIqVeC/R6/wAnVDsLT3KKtkHKYHXx728nIOo2/wDst17JYVObwNPMpFVUhvTgcFaVZ7SEHKBVhUCrAgVEqZFlFaRt9EJOS0qoDudIWnraV6WXxKiRth4r3D0ryWAv5LH6F/CdvpNvWvZ18ThiVS0N2SOPpXq05/FxtHtjtcbe2altKkyDWJBIBG0FZkVE0PBOtZxIyG3mVtqRCRWZYrIJZCNVt+CzocGqHtDnNDR/eW7wGkilfPFJEOWZGC0k3tvy7VmQRsEUklRFICcmAu1b84Xi1fIvE4q+l4/jaVq7ry89+THwvDXXzvew2Z8+3cVtKPBnzxB749SMm5kkcQHDmy6di2URpYCxkEPLzD9pI25vzBZAgrKhxe8udccV49Xy4j1M+3SPExOZnEK6ekpaZnJQx8sRtLhZvZ3q513OHKODiNjQbALFlbNESx12gbQhpFxqnPpSt93t7K+PWsem0onMbONdwbcbAtiZ4mghp2C+XX3LRQQudI21zs27+ZbghkTb5Od7e3avTSZmHh8jSruzLIa5guXXtz9NlTU18VPCXZRstfWO/YsCuxGKjjLpXXeM9S/39g7F4PHNI5aqRzWPvbIcAvZp0nuXztTbHqrYaRaVFwdDAbA7r5npXjJZHSvL5Dmc80nuJcXvJLjvKqc8gLvn6corgnO5yqHuTc6yrcbrGWkCVvNH23p5v8Y+5aNeh0aZelm/zB9yR2stuxqyI2qLGbFkMb6VtzSY1XsaosYr2M2IibG7FkMaoMar2tRE2hXNCrYFa0IiYU2hRCsagm0Ll3hXdrYxSN8mEntP4LqbAuTeFJ+tpHG3yYG/eUt+stV7h4jVQGgm2xNI55LzS7szGXWxF0AyZA1sbBwAAWCVsZGHFWxyQlpqw0NkiJAMlhk5t9pttHMsb3BWufqCjqC7hyLu5c4n00rpC/3bByd9cSstb/EFLEQPyhUFtrco61ulZkUX5KcZpi01YBEUTTcxnyncDzLXSjxC4uBJvcb1M+z+MzDbtwapd5UzR2A96pV1JlgI/vTuPYB3qm6n9loJt2pJoOy6Jw8hovh7LWPIgnrzW4CxMLi5HCqSK1tSFjfQFlr4t5zaZeyOghCFlQE0k0AhCEFSEXzQsKFGVnKROaf1hZSRZEcTqo+RqZYyPiuLewqlbTSKHkcerGWt+dJA6c1q7L7FZzEPLPaJV8A16atj261M49hBVKyaAa9QYh8aVj2drT61uO0aihPiOHAq8rFoidd445rKK1btIRKjvUionakCLs1Gykiy0L6B3J4hTv8AJlafSF06soDLicxEYfyhBtrAZWHeuWw+LMw8HArtzKSOanZPJNyTHta7xLlzzbhsAW92KSzFZtbENLFAQwGMNkaLEsLD4x9f4hbemwd7I2yTubGCCDygJdnwF8t5CyopYoIwykgDM7F1wXHpPG/BMNe8h7ze4uSTmV5b6r208We7CMx09m0kdsrF5HjG6pqIy14Mz8/SVmA2YeQDXOGy59uZWxR0xLRJA6aYN1nOOxp614PK8qNKsTjOXs0610v4rwmnbK8ykWYzLVtmV6KnkiYdVzmg7rleYE9RC4NgBZq7HBtxbgVXN7sqp+Uc8j0ZL5uhp6+r5HNj0mto8s/lbENpjRh90B8TwXHa0FY0QhIvLGctuSxTCQ/Wc4m4WfFAzkuUlOqwZ57/AGuvu6Glf+rN6aVIiZ6E9RBTU5laXBjd1r58F5iu0krZZhyDnstkyNmZ61nOxk1WPHD4gG08cZNhtcbjMlafEqsU1bOyKMcsXZSW+KLbl216zSO3q/5vHrZnblgV9fW4hVCjia90xIaWgZk8FjYho9ieFwcvV0j2Mcba9wQDwJBy61naNyTnSpjoHw8rd2rypyebbL8TmFvp2CPDK2r9x1mHci9j5YKh2vDUEO+KL5r3UtM1jL855OI1rRHWXPXAk2spUtBVV9Q2npoXSSu2NG1dFNBhNBVQvipYaluL1LJIY3AAMjA1iBfZ4xt6FuGQxQ4lQ1EVPDDI90kVnwCOQjVJAA2EXG1ay8+5xl0MgJGqcsjkoCB7h8UrslFT0xo4A7DWvM5casNhZYPvmHEm7bLApp6WlnwXD4KSmdT1TJhJrxtcXButbPqTJucokhfH8ZpF+Zeh0Wbejm/zPUtlpPVMxLRSirpYYW1BqZYtaNgb4o2CwWHomy9FP/mj7kjtc+m6YxXMYpNjVzI10YmSYxXsamxiuazdZEDGq1oQ1qsa1VDaLKwJNapgIJNCmAogKwBETYuQeE1+tpQW+TE1dgauM+EZ+tpdUDyWtHoWb/q3Xt5QoTUoonTSsiYLue4NA5yvNL0IBpc4BoJJ2AC5KzHsxYRnXZXBm/WZIB9ytknNOXUeHa1xflJWjx5CNvQOYKp1LXxCKUCUOkaXgtLtYW2rlMk3rE4mWG3I5KE7yYze2Qtssti5wr6SSV7bVMABLxlyrL2uecXGe+/MtZUEcn1qx21PTYt8TAqMeUXu+1b1LHyWZVgMoMPjG6na49ZJ9aw1mFAVtMzlKmJnlva3tIHrVS2OAQ+6MfoIrZOqGX6jf1JacRKx27XG3Vja3gAFJARdfFnt7AE0IUBkl0JoQCEIQUqSSAsKEdiLoG5By/TWHktI5jue1rvR+C86V6/whxFuK0826SG3Yf8AyC8gV9XRnNIeW3ZK6geGYhTuOQ5QfeqChr+Te1/kEO7M11ZYIi9z4jNAM9R7mdhssglPFmCLSOpDcgZSe3P1otnnsW7MobRxSOa97URNODUJo8Kp6kck0hppi+176xuFotKotUUUrqdsEjmOa5rYuT+KQBl1rnW+Zw+fo+dy3iu3GXnUAKSAur6IaLFduwqN9VhdC9pa0Phbdx6AuJgLs2jEjpdGqAx07pXujDQ4EeLZZ1ZtGlbb23pW26kS2L4GRMEcdnSOyAaMgpNgqmPELowyw8dxOtrcw9t6tk5WiiLCeUmffVIF9QLIjJLMoWmUnxjv6V8mtL607Z7e3U1prXd/FFPyMNS3Wc7JxBBbkfbirayI3cIhZruCQgaHGTkwMrZm6lBOwlzRYnZdd/G8OdOsxqe/bHNGpfNWPFGQ7xzn5I3qwxOfqgbSdyujgMklxa9806mripGuDbF+93BfTppTb1HTlqa8af8AsqpRFSt1prFwGTAvOY3j+o11n52sANyx8axtrA4a9yeJXkKiodUyl7zluC9la104xDwWvbVnNmbh+MSUWJmt5MSXBBaXWRi+Ktrah8kEbow/42sc+gWWtLhZVufzrlakW9y9On5GppVmtJxlMSujcHNNnDYQrpcYrKh0YqqiWoYwg6kshcOjMrBc7nVZdmtvPPtucWxubF6iFzIWU8cDAyKKK+qwcyxZqzEHSsdJPMXtPilzjcdC9DonyeGaPYnjjYWTVMLmRRBwvyd/1vSt3glcdJKSnrK+CP3TQ18IbMGAa7XH4pTLEvANqq48oxs0p183jWOfSqHVE12/nX+LkM9i6NjzGYDhWIVWGBlRPU1D46mdhH/Dgn4nXfauYudmSix7TdK9zdUuJaDe116zQ8a1BUH+b6l4++d17TQtt8On/wA31BK9lunoWM5lc1ibW2VrWrthyyTWK5rUNarGtUQNaphqYapgKoQCmBzIAUrIABTaEgFNuSCbQbLiOnz9fS+t5nAegLt42LhOmT9fSzED/NIWL/q3T9mjWZhBAxSC5tfWaDzlpA9JCw7JgkEEZEb15JelsMEdCzFoG1ERLjKAHF1g07MxbPP7ltsQhqsOoqs4hVtqxO8BkbJCQDfbzcMlppX0teeVfIKaoI/OAtJZIfKyzaTvyKg2jo2HWmrWFo/VgY4uPNcgALlMe3l1PGm+puz6FK3Uo6uoLS1j28ky+8kgnsA+5ayp+KBzrY1tX7pLWxsEcEYtHGDew49JWvmGtIxvErUPU22KkCeOMbI4Y2/ZCwllYm6+ITW3Ot2C3qWLdSOmpC9BoPDyullGSMma7+xp7159es8HUWvpC+T5OB3pIWNScUlqvbqCd1FNfIw9ZppBNA0JJqAQjNCCi6LpIWFSuldK6FB47wiQ61LRzbdV7mk8xH4LwJXS9OouU0fLj+zkab9OXrXMyvpePOaPPqdkUiARbcU0ivQ5q8YdrYlDMRYywxvJ6Wj1gpXTxkHVoZdxh1fouKiM2hdLdQykJ5WgBsrwBuDioue55u5xcec3WwwnBavF5wyAMay9nSPcLA24bT1KGJ4PWYVO6KojyFiHtzaR0rGYzhwjV0Y1ePMbmCNiYCVk1t6TC7J4PdWo0WhDj4rNZptt2lccC6r4Nq+CHAnxzSBgD3AX7V0rG6JhzvMx7epfRmoa2Fsjw1m0g2PoWVEHMeIzrEAWu7NUx4lQxXInbfapHGKBpuJ2jitxpTnpx3Ng5jTHY5ZbFhxUkbNZ7vFaduaodjtCL3nbbhcLXVmORS5NniA3AvC710Y7krq2rExVn12JsijLIjqM47yvGY1j4aSyN1zssFKvnkqLhtdSMB4yrRvwpjnl0mLUVz/MXafUYhmPc5lgSzOmfryG5VRes92F0w+NjNEP9Sg7DKLfjVIueHSJhgOfkqy9Z5oMOHxsdpexVmjwj9bHqfqas4MwwHOUNZZ5pcF349F1MS9zYEP46D0RFMLlk4HpBUYK+QRtjlhmbqywyjWY8c4WfV6aVT5KYUlPT0tPTyiZsETLNc4b3cVpxDgI/jTj0QlPU0ft/a8p6ISmGZwzqfSyugq66fVie2uDhNE9t2G/NfctE51yVnaujvzrOeiA9yV9GvnOqPRAe5MEYhg62a9zoL42GVH+d/8AULyl9GL/ANpVn1H/AIrdYLpLgGD076eGqnkD3axL4jw5grWMSW9w900BWtAXlRp1g4/av+gUfCBgzXWMkt+aIrrmPtyxL1wsrG7F48eELBQQC+b6oqY8IuBtOb5s/wCUUzH2Yl7AKYXj/hFwJvxpJvqip/CNgI2yy/VlMx9piXrwpDYvJfCJgQGc0v1ZT+EXAGtvy0v1ZT0mJetFlK68iPCPgFr8tLb/ACyn8I2AkXEstv8ALKevtcS9cDYFcE0lk5XSOvdxnd966YfCNgRaSJZfqyuT4hO2pxConabiSRzh1lctWYw3px7Y4UudRCkLW515Jl6AAXEBoJPMm5jmGz2lp4EWXt9E6WkgwuGo1mNmqXuaZXAEttsaL7CVlaS0lPNglU+YtkfDYwykDWvvbcbVwnU/LD41v+rEeRxbfXTnhUadokxSlYdjpWD7QUip4UA7HqYEX1SXdgJXWH2U612tVzO4vcfSqU5DrSOPEqKkdKd17jwZxXqq6U/qxsHaT3Lwy6N4M4tXC6yYj484aDzBo9ZK5a8/hLpp/s9tdO6iEL5j0p3QohMFTCpXTuopqYEroUUJgUXSugnrSXJUroUQmg1WlEPL6OVrRm4Rlw6RmFycnNdnq4+XpJovLYW584XGHDVJbwyXu8WfUw4aiJUSpKJXrchirQ7B6OQbY5ZGHrDSPWqIzeJp5lk1V34JK2+Uc7X9oIWJTm8LV1/8p/W0wjFThNSJm08UpuDd4zHQdytxnSGsxh5DyY4MrQtcdXr4rVoXPbGcuE+LpTq8sx+RWTshNaekBTbLIwWa4gcxUEXyVicJhb7oktm4nrUXSPP6zu1Qukelbi8piFomcMtYg7s1B8pvfWOarJUC7nWomUxBve4naqy88UnFQc7NaiZZmEi7fdLlHW25KF0rqiWseKWtzqN0KsrGB73hjGlzjsAFyVJ8csZIfE9hb8bWaRZbqOnOGaKDEIzq1NY/UDwbFjM8h02VEeLOqdHp6ComDpGysdEXnMi+YvzbVnd9NYarWS1+dbIaNYqXOApwbM1xZw8Yc3FY/wCSazkuU1G/o+ULNYa+p5Wrtsruj7TEqoIJ6l5ZBE+RwFyGi9kpIZob8rE9ljbxm2z9it1jEIwrAcPportfVAzTuGRccrDoF1jz102LYTQUVzNVRSPjDdrnA6tu7qWYtn2uGpumHLPjwGslfqxuhfZ/Juc2QEMdwKsk0cr4xOHGLlIGl7ohJd5aNpA4K7oTEtdrHijWVV0XWkW6yRcq9ZK6ot1ilrKF0XCCesUw+yrui6C3XuVIFVAqQUyLQVIFVgqYWJlqITCaQKaw1hsMMxyswnWbA5ro3/GjkbrNPOpYrj9bi2q2dzWxt2RsGq3sWtRZZxGcvPPjaU35NsZRJV+DG2JzSW/RwSHo8W3rVDldhTtVuISH5HVHW4BX+S7/ANVu2pIKFQLqugMXJaLROt+kke7pzXKhmuxaKxcjoxQM4xB3bn615vIn8MOunHvLcIuldC8GHoSumFBMFBNF1G6d1BIFCSEFCR2oQVwaAUlG6LogOYK47isXI4pVRAZNmcB2rsS5VpVFyOkVY2214d2gH1r1eLP5TDnqdNMkjemve4JEB2HVrD5DXdjh3rCpDeG3ArYU7ddlRHa5fTyWHOBf1LWUj2ta7WIGa6R7qk9srciyjysfljtRysfljtWcS1k01Hlo/LCOVj8sK4kzCSFDlo/LCOWj8sJiTKRSJUTLH5QUTKw/rBaiJQyVBxuLXQZGbnBQL28QtRCSHG+wbVUTmpkgi+sFA7ciFuGJK6W1FjxCVucdq0guldHWEW5wqPU1cgqtA6VzP3eXUfzbR6wqcKhoJtHq2rloGOlpGixLnWffitTh+KSUDJYS1k1PMLSRP2Hn5iskY7yVFLQ01LFFTTCz2FxcSbjO/VZctv8AGst1i1fJHX4IxsjoozAwP1Da4cQCPQjEMQpcM0tmmNNUSz31A0PaGG4ta1r7FocSxl2JRRMfTQRmFoYx7Na4aN21Sfj00jWvfFA6qY3VbUlp1wOPC/PZIouW20ukFTh+FVcYsx0bm24HLJR0MpojUPq3n84GuZEN19Uknp2dq01Niz4KU0kzI6qnLtYRyg+KeIIzCjJis3LwywalMIDeNkQsGneeclNs7dqZ95ei0KcA6vMmbCI9vla2SyKZ5fprimsSbQyDPhYLzrNIqqJwMLKeIB/KOa2PJ7uJTj0jrYq+auZ7nE0zdV7uSGY/FSaTmZXdDVB25F0PcJHl/itub2aLAJZeUurmaLpWHlJ2HlKg1kXSy8r0J5cfQigFMG6WXE9id2jeexBIFSBUC5rTvBHMgPaOKguCsBWOJW8CpcuBuKzMLDICmsX3UAfilSNUB+r6VnEtZZCFje677GX60/dDzsiKmJMrXK7DT/y6tPlPY37z6lhmSZ2yBx6AVnUkT4cGe57C0yT2zFtjfxSeiO1CChCBEkNNttl3DDYhBhtNENjImtHYFxWmiM9VDC0ZySNYOsgLuLQGtDRsGxeTyJ6h10v6ldO6imvG7HdO6hdSBQSTUUwVMB3QhCCm6V0IXmbF0XQhA7rnWn0HJ43HMMhLCOsgm/3hdE2LxfhDhvFRzDcXNPoK9HjzjUY1I9PDIWXheHuxTEYqNjwzlDm47gF6au0WwyCi1qKvkfPnra7MjbrX0JvETEOGHlaKdtLWxzSBzmNPjBu0i1lX7kwXhX/7aruTe+0G21JbzMItFLg18xXf7aPcuDbhX/7aqSVzP2Yhd7lwbf7v7I0e5cF3+7+xipSTM/Zhd7lwb/1/2Ee5cG/9d9hUpXVzP2mIXGnwXhXfYS9z4L5Nd2sVBUSrEz9jI5LBfIressS5PBvkqz6TFjFRK17+0ZRbgo/Y1f029yV8GH7vVH+o0epYZTjYZJWRggF7g252C5V/+ozR+Rz+61P1w/7UiMHGylqfrh3L3cOA6P0erRTQ8q9wGtKTmeNl4PF6aOjxapp4iSyN9m3222rFLxbpqYwL4P5pU/XDuS1sG81qfrh3LBJzSXXDGWfrYN5pU/XDuRr4OP3Kc5b5/wAFr0Jgy2AmwgD+zpT01B7kCpwkfwt56al3ctehMGWw91YV81H/AOS5Bq8K+aP/AMly16EwZbD3ZhfzQOuoen7swu39jt/+Q/vWuQm0y2Bq8M3YPH9fJ3pivoBswen63vPrWuTKbYMto3FKIbMGpOvWPrVsWIxyEiLBaJ1tv5q6066FoXHSUuCtq2wsmne4tfrC5GdrLnqTFIy1XMzh5N+LQtcQ7B6EEbuRsoHFYDf/AJVRD+kt9p+aWaakqY6eOGZzS14YANYDeRxXj8lqsRMZScxLZDF4Nn5JofqlL8rw/NNB9StWApK7YTMtn+WIbf2TQfUhMYywCzcNoB/QC1drphNsLltfy24bKGiH/t2qX5fn3UtGP/bN7lqRtUtqk1gy2o0gqt0VKOimZ3I/L9du5AdFOzuWrTCm2Fy2Z0gxG1hLGOiFg9Sj+XsT3VRHQxo9S1yamIGa7GcSec62bqdZQmr6mqhDKieSXVN267ibdCxEwriBfTU01XJycEbpH8GhTrsOrMOkYysp3wueNZuuLaw5lu9EKyKnE7RYVDnCxJsQ227rWdpdi7K3C4aeWobPKxwLA3PUG9Y3Tuxhcemh0Zh5bSTD2fzmu7M/UuxLlWhEfKaTwHyGvd6PxXU15/I7dNPpJNRRdebDqaajdO6IleyRcRsSugouRd3FCXSUKYAhCF5GwmkmgF5nTuIPwNslv0UzT25etelWvxzDnYrhM1GxzWPeBql2wEG66ac4vEpaMw5RS1MtHUtnhNnMPbzLbVWkpmpwyGn5KQXu/WuBfgth8HuIn97px9LuR8HmI+e0/Y7uX0N+lM5y4bbPJ7MuCS9b8HmI+eU3YUvg8xHzym+0tcun9pss8lZC9b8HmJed032u5L4PMS87pvtdyctPs2S8kUWXrfg8xLzum+13I+DzEfPKbsd3K8tPs22eRKS9afB7iI/fKb7SifB/iPndN2OVjVp9m2XkyFAhetOgGIed0/Y5R94GIed0/Y5a5KfabZeSKiV60+D+v88p+wpHwf1/nkHYVqNSn2m2zyBSzGY2r1x8H1cf3yDsKXwfVvnsHYVrkp9pss1bNKa5kLWWjc9osJC3NaiWV8sjpHuLnvN3E7yvWfB5WefQ/RKfwd1nn0P0SpF9OOlmtpeNJuUl7L4Oqvz6H6JR8HVX59D9ErXNT7Z2S8ahey+Dmr8+h+iU/g5qfP4voFXlp9myzxiS9p8HFQf4hH9AqQ8G8+/EI/qz3py0+02WeKugr2o8G8vzgz6s96l8G79+IN+rPenNT7XZZ4e6a9wPBufnEfVnvUvg3vtxH/b/ABTmp9myzwl017v4Nm/OX+1+Km3wbR78Sd1RfipzU+zZZ4MLLo8RqqBxNNM5mttG4r2rfBtT78Rl6mBTHg2o9+IVHU1vcpOtpysUs8HU1c1XLyk8he47yVSuifBtQb6+p7GdykPBth3n1V9juU5qHHZzlNdGHg2w3fW1f2P+1Sb4N8LG2rqz1t/7U56HHZzgBMBdKb4O8HG2WqP+sdysb4P8EG0VB/qlTnovHLmQUgunjQLAt8U5/rOUhoJgA/d5j/Xd3qc9F45cvTC6mNCMAH7m49Mru9Tbobo+3+HtPS93epz1OOXKU11kaJYAP4bF1k96mNFcBGzDIOw96c9TjlyNGS6+NG8Ebswyn+hdTGA4Q3ZhtMP6QU56/Rxy46MjcZEbE9a+03XZBguFjZh9N9U3uTGD4aP3Cn+qb3Jzx9Lxy8J4PWa2OyPtfUgd1XLfxXSljwUlNTOJgp4oiciWMAurgvPqW3zl0rGIwaaihYVK6LpIuoHdO6jdCB5IR2oUDQi6S8boaajdO6BE5oRvTQCE0lQIQhA0IQgEiE0iqIOVZVjlArcIrKgpuUF0hCKiVIqJW4REpIcldbEkwo3TBREkii6V0BdSUbpohoQi+aBoSTRQhK6EEgmEgmEEgmo3QCgkmo3TuoJXQop3UU0JXTuqGmooQSuhRTugkhRui6IldF1G6Lq4EkwVDWTBTAldCjrZIumBK6FFO6YDui6W9F1cCV0XUUKYEwTxQobUJgTui4QheB0Fwi6EIC4UghCAui6EIApgiyEKguEXQhFK4USUIVhEXFVkoQtwiBIUboQukJKJKiXBCF0hECUroQtILqQKEIDWyUdZCFQwVIFCFEO6MkIQF7IuhCKV07oQqh3TuhCKd0XQhA9ZAchCgesnrIQgNZPWyQhAtZPWQhAayLoQiwNZF0IVQayLoQgd0AoQgesjWQhA7ov2oQgLhGshCAJRdCECuhCEH//Z</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -453,7 +459,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update inventory — 04/08/2026, 7:24:31 am
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,7 +422,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>box01</v>
+        <v>B001</v>
       </c>
       <c r="B2" t="str">
         <v>New box</v>
@@ -434,39 +434,19 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>2026-08-03</v>
-      </c>
-      <c r="F2" t="str">
-        <v>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/4gHYSUNDX1BST0ZJTEUAAQEAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADb/2wBDAAoHBwgHBgoICAgLCgoLDhgQDg0NDh0VFhEYIx8lJCIfIiEmKzcvJik0KSEiMEExNDk7Pj4+JS5ESUM8SDc9Pjv/2wBDAQoLCw4NDhwQEBw7KCIoOzs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozs7Ozv/wAARCAF3AfQDASIAAhEBAxEB/8QAHAAAAgIDAQEAAAAAAAAAAAAAAAECAwQFBwYI/8QAUxAAAQMCAgUGBwsJBgUEAwAAAQACAwQRBSEGEjFBURNhcYGR0QciUlShwfAUFhcyU1WSk6Kx4RUjM0JDREVjgzVicnOCoyQlNNLiZISUwqSy8f/EABoBAQEBAQEBAQAAAAAAAAAAAAABAgMEBQb/xAAmEQEAAgEEAgIDAQEBAQAAAAAAAQIRAxITMQQhFFEiMkFhBUKB/9oADAMBAAIRAxEAPwD1haNYElMpH1qS/NPpI2CVgVKye9BEAIsE0IEQjVFk0Khao2ILQmhBHVCLDbZNCBWTAQkgLDelbgLppKgsBzEcUAWzR0A5IOfFAWF89/Ynluub5bc0iTvFudHbxzCIMri5358yGgNO+wz22si5ve23Pbkjq9KB6oN7dpICPFGTr7EA57r223Rewt6UDs3Kw7c0ZjLLI5Z70gee6Bfbs6QiF4t/i3tzbPQm0eSCehFjsIJPOjLe6x32zQMAEi9jwuUrNJ2bdvEp34jdlxSu7abdKoRAGW9FrA7OxMWDhsPMgEm4I699lQiPFsdnC21GrkQBkO2yNYtO/PNAB29mSAI32uiwtsAQi/EAooAvsyT3XG9K/MLpoAgbLIIyQjqQLehBzQgE0k0AlZNJAW5kWQhAW6EWbwTJQDuVQWvtStY8UztvxSvnfNFMNtcbPX7XRqttmL79qMzzX9ro5gLqofi5HbY5jilqtzG4JnMbALozFs8r9aoRA1bC3EJhtrnxb7jvRtabCynrPubAHcbjYUgBIsA5otrXz9KQaB4xuC3cDZIWLsibeTe9ky0EnVPi7s1Q7AHYAbZpWaWgEtDto5kr5jVeSU2nK1za+ZKZQODgfFcWjhdCkDrZl4H+J1vUhX0K3fFKkk4ZFA2LzNhNCSAQhCAR1oQqBBQkgEIRZAkJpIBJCFQ8rdCVs+KYF8uKSAujj6UXuANlkXy2nPaOKINhG870gL9CY4bkr2tvVDsBfbzIPEX2I2ZJAAgiyB2y9tqedja+e07VEHPcn07uZEAIG0cyeRve3WkObZfJLabceZAza+7qQTfK/TlZHMf/AOpXtvNt6BngTYHpRkQN557qJ6kHoFuCoOfLqT2brZJW3HbfsT3Dh0oADaPQjbwSG1PcEUxkhGYPBLtQNCSEDQkmgEIQgDtRfNCEAhCEAmD0pIVD27ckC1yL7SlY2zQgYzzJtZF7hG7JA2WyVQwXGwtlsQTexyy2JXvmSSd90yLm3P0ZoHfmJyvmEtpF+G8pGwGVwmAA7LdzKiWdwbgDddIiwtY3323XUQDfIjiLm10zttnt3FVDvck26bZIPjA2vnxQNhte2642oBBsANp3DMqKlrMZkWNdz6pQlc/qkt4gcUKgSGxNILztGhCEAhCFQJbNyeaRQCW5BQgEISugaWaEkDRwHYkhUOxI2FLPZdFkelAcyXrRmEA250QFF89pQhUHVZHPvCPQkMige7m3I3bfSlu3J57EAb32Ivlnmltz9SPvQFwRmjZlstxzslnnvRf23oHfKwKLi+ZUev8ABF7EKiVxxCD2JXPoRsRD2o9tqE1AbkIR7bVQAoRdCKaSEIBNJNAIRdCAQhCASTGxF1QZ238EZ70IuqA7b8UwSDcXBS28yOfeUQHp7U8srZbkHK6V78boHsIzsUbwbXuOtF87WHajPs3Kh7MjccbFDbHIm18kjYZ52tndG8gEX4IH1m6Dq5ndfednSle1skwdU7L7rIES3e25G9CbSQMnDsQglcAEk2AC1xx3CWEk4lTW3DXCzZBrRuHEZrjVbGYKyaI/qSOHYU0dKNTOUvba6udIsFH8Tp/ppHSXBB/E4PpLkN0wV6PjV+3Pll1z30YHfPEoO0qJ0pwMfxKH09y5OhPjV+zll1b314F84xnoae5I6XYCD/aDfoO7lyq6RV+NU5JdU992AD9//wBt3conTDAfPj9U/uXLErp8apyS6idNMCAyq3E/5T+5I6aYFb/qZCf8p3cuXphPjUOSXTTptgY/bSnoiKj798E+Um+rXNbpJ8ahyS6WdOMF3OnP9P8AFI6c4MPOPqx3rmqLq/HonJZ0g6d4R5FSQf7g71E6e4OP2dV9Ad651miyfHoclnRTp9hG6Gq+g3vUTp/hI/YVX0W9652kr8ehyS6H8IGFHZT1X0W96PhAwvzap7G9650SAi+afHockuiHwgYZupansb3o+EDDh+61H2e9c7Urq/Hockug+/8Aw+3/AElR9nvT9/8Ah3mtT9nvXPboup8ehyS6F7/8O81qfs96Pf8A4b5rU/Z71z3WRdX49DfLoJ0/w3zWp7G96R8IOG7qSq7G9659dRJT49E5JdB+ELDfNarsb3pjwh4Z5pVdje9c8ui6vx6HJZ0P4Q8N80quxven8IeGeaVPY3vXO7ounx6HJLog8IWG+aVP2e9P4QcO81qfs9650mnx6G+zovwg4b5rU/Z70vhCw63/AElT9nvXO0XV+PQ3y6H8IWHeZ1P2e9MeELDvNKntb3rnJcgOuU+PQ5JdHHhAw/zSo7W96fwgYdfOlqLf6e9c7undPj0OSXQ/f/h3mtR9nvTGn+HH91qfs9654DmpAp8ehyWdB9/uHea1PY3vUvf7hvm1T2N71z29kEp8ehyWdDGnmF/IVX0W96Y07wo/sar6Le9c8BTur8ahyWdDGnOEnbHVfQHepDTjCPIqvqx3rnYKYKfHockuiDTfBz+rUj+mO9SGmmDnzgf0x3rnV00+PQ5JdH9+OEH9acf0/wAUe/HBvlZvqlzoEoyT49Dkl0b334Lf9NKP6RT99+C+cSfVuXOFHWU+NReSXSvfdgpP/Uv+qcn768F86eP6bu5c1BKd8r36k+NU5JdXocTo8SY91JNygjIDrtIsTs2rKyJ2ALzOgkdsMnlP601uoAd69P0/evHqVitsQ61nMA7Eb+CezpSGef3rCg557UJi+6/UUKgIuCFyXSWHkNIKxlsuUuOsA+tdcXNNO4OTx/lALcpG0/eFrxp/LDOp00uF4XLilVyMbg1ozc4i9gvRVOgc7cJGI0NR7oYRfVsLkc1lqNH8QjoKtwmyjlGqXcF6iXHIcIp9emqGMgF9WzruIz29q9N5vuiIcoiJh4QiySGyOmL5SLB7iQOZNdpYRSJTSKBJIQqBNRTQO6LpIVDQEkIZSukXKKLoZSukldB5jdB6jANHaCTD2Ylipc6KR3iMa6xte2xWaT6K0NHRyYjhE2vTxODXtJ2X9tipwTH6FuEtw+teIponExSOGVjnkdxWNjmkDKikdQ00weJXDWaz4oAN7nnXGsX3+2/WGh2IugqN13YSLkaygSldMCzWSLlC6LpgSLkrqN0XVwiV0XUboumBK6AVG6YKuBIKSgCpJhTCHZBCCLhVHrsG0Yw0YO2vxV7i6QBzIwdoJ3Dm2lYGlOjkGDspK2inbLSVYOrY31SN11dh2lcMVBBT1DjFLDGYiS24c3ZcZHOy12OYx+VHxxxlxgivqlwtc8w3BcNOL7p3NTjDVgp3UdiLruzlO6YdZQTuqZTundQundDKd0wVAFMFBMFSUAVJBIFNRumFFSuU1FSagYC22jOCw41XPE8wip4ra7t1zsC1jWgqWFV82ETyxSxSOilcDrMBNj1LF8zX8SO3qa/RzDpsNqZqImOWmFyLEAjZnfevHjavQ4hjkb6d0dMCXyiz3lpH35rQBuaUice1l0TQ2PU0eYcvGe53pt6lv8uZarRmPk9HqP8AvM1u03W16sl83UnNpeivRXz4oAPDNCe1YU9Vx2AlCWqOHoQgkvB+EOH/AIilm4tLfSO9e8XkPCBFehppLbHkdo/BNGcXhL/q5+gNadrR2KSF9J5jtkkQdwv1J3Up3uGB1wa9zc4j4ptca1j96sRmcCuzuB7CkWngexYNES+C7iSb7yr9VWYxOBcWngexLVJ3FUlqWqmBfqO4Jhh4ekLH1EtQcB2K4Msrknc3aEuTcOHaFjag4BGoOA7FcGV5Y7gO0I1TzdoVGoOA7EanMEwi6x5u0ItzjtCq1BwCWqOCu2BbmNjh2oseI7QqtQcEiwcE2i7UuLHVPWExHq7A0dBCxiwcAoFg4K7Rllp5u0KJa7gO0LE5MKBYOCu0yzdR3AdoS5OTyftBYOoOAUSwcFdqZbDkpPJ+0E+Rl8n7Q71rdQcEaiu0y2XIy+T9od6ORk8n7Q71reTCfJAptMthyUnk/aHejk3+T6QtcY0uTTaZbLkn8PSE+Tf5PpHetbyfMpiMcE2JlsBG/wAkdoUtR3D0hYIYOA7FNrBwHYm0yzNR3D0hGo697DtCxg0cPQnYcAphcsmxtu7Qkedze1Y9glqq7Uyvs35Rn0kWb8rH9JUanMjV5kwZZFm/Kx/ST8X5WP6Sxw2+5PVVwZX+J8qztQHM+UZ2qjVRqpgyyQ5nyrO1MFnyrO1YwCkGqYXLJuz5ZnanrMB/Ss7VQGjgpBt+CmFXa0fyrO1SBZ8oztVIaFLUCC3WZ8qztTD4xkZo7/4lTqjgtXiX6YDg1Igy9CWvjtcbQCOhTbOQ2ylXHk6kxtyDGtb2ABYussQq15vmoXtnzXUdZNo13BnlHV7UkdYwqHkMJpIsvEgYPQFljnzUYxqxtblkLKS+Tbt6o6GSEdqFlRbmQn0WQga85pxFr4AX2/RyNPq9a9GtVpNDy+j1Y3baPW7M/Us0nFoLdOTpJnaUl9V5Aro2iSgxCMi96ZzgP8JB9SousrDfGqnR/KwyM7WFajsaTDnXjeOdZq1+HHxnhZ63fsjokIQshFCElYhDQhex8HOHUGJ4lVRV1LHOBEHNDxexuulK7pwzM4eOsiy7qdE8AH8JpvoJe9XAPmml+rC7cP8ArHI4WhdyOiuA/NNJ9WEjotgOz8k0v1YTh/1ORw09CRXcTotgPzVS/VhROi2A/NVL9WFeH/V5HDiSoOK7idFcB+aqX6CrOiuBfNdN9BXhORw+6g4ruJ0UwHfhdP8ARUTopgHzXT/RV4U5HDr2UbruDtEtH/mqD6JVbtEtH/muDsKvFJvcTui9l2o6J6P7fyZB2HvUfeno+P4XB6e9OKTe4ttKkF2f3p6P2t+S4Owp+9TR+/8AZcHYU4je4uhdqGiuAfNcHYpDRXAPmun+inEm9xQKY612waLYB810/wBBTGi2AfNVL9AJxG9xIA86mAeC7a3RfAPmmk+qCtbozgI/hNJ9SFOI3uHgHgnnwK7mNHMD+aaP6lvcpjR7BPmmj+ob3JxHI4TY8D2JXttyXe24Fg42YZSD+g3uVjcGwsbMPph0RN7leJOR8/GZg2yNH+oIE7PlGfSC+hRhmHt2UdOP6Y7lYKCkGylhHQwJxnI+eBNGD+lZ9IJiRh2Paf8AUF9FNpKcbIIx/oCkIIRsiZ9EJxnI+dQL7BfoUuTfuY49S+ixDF8m3sTEUdviN7E44OR85kFpzBHSEA2Xq/CS4HSt7WgANiYMuteTXK1cTh0rOYysBUgq27VYFzluEwpKAUgsqa1k7OXxOOLbrPa3tK2awKNnLaQ07f5zfQfwWoSW6xBwNdMRs1ysZTqH6873cXEqsFYiPTSV1k4azlcTpY9utM0ekLFK2ejcfK6Q0TbXtLfsF/Upb1WSO3VSjnvZMDJC+Q9QQiyLZKKLc5QixQgax6+PlaCeM/rRuHoWQovzaQucdrLirxZxCgsmvjbDWTR53bI9pHQSFjFfXj3DyT2Svw9+piNOf5jQegmx+9Y5TifqTMf5LgVqBrKccnXSx8CR2FZyxq0CLH6po2cs+3aVfrLpftmElElInNF1hTuldK6LrUIkF7PwYS6ukkjNz4HfeF4u69T4OpeT0tgHlse30Ltp/sxbp2VyipHYokr1uCJUTdMu51AniqgJUCbBDnKsuQNx4lVudYIc7JUverAk5ygX86rdLzqp0nOqLi9QMmeaoMnBQMmSqr9eyXKcVjGXikZBxUGTyme1PlFicpzpiS29BliTnUg9YYk51NsiIzGvzyKsa9YQkVjZEGa16mHLEa/LarGvzTCMoOyUg5UNdzqYcoLgc1MOVIcpgoi0FSuqwVIFRFgUgqwc1MFFTT3KIKZPinoQcU8IL9fS2q/u6o9AXmwt7prJymldcb3tJb0BaILhqfs706SCsCgFNcZdYSCkoBSWVBOSxMHGvj8bvJc53YCVkuNgVj4E0uxKZ9/iQyO9XrT+Sk9sxx8bNAKTjmelK6ipXW+0Mj5TSSE+Qx7vRb1rz+1eq8H8WvjE8nycGWXEhc9WcUlqv7OhppBNfJeoIskmgEIQgEEW3oSXJXJtJouR0grWWy5UkdYB9a1K9Jp1CYtIHPtlJG13q9S80V9bTnNIeW3YKSEl1RRjIAx57gLB7WOHWxp7073CnjxPK0M+Xj0rBfnBIKqB8ULpPUM/0yUrpEpXWcKlfNF1G6LrSJ3W90Jl5LS6gN7XkLe0Fefutjo/PyGkFBLs1ahnpNvWulO4Yt0+gL+KoFyWtdoUC5ex55MlQLski5VuciG52Src7NRc9Uvk25qiTn2zKofJzqL5M9qodJzqqm9/OqXSc6rfIqXSZoq4yc91AyLHdLbeqzKgyTIomQLFMqiZedRWWZQjleKw+VtvRyt0RnCUKYk51gCXnUxKhhsGyKwSc6wGy86tbIiNg2S6ta/isBsmxXNkRGe16ta66wmPVzXoMoOVgcsZr1aCiLw5WArHDlYHKIuBUwVUCpgoLApHYqwVJ5swlIHBtJ36+klc7jM771rAVk4xKJcYq3g3Bmd95WKFwv29NekwpjYqxZTC4y3CQKd1EFO6y0Uhsx3QoaPs/wCumv8AFhDe1w7kpzaF/QrcDGrhldJ5TmM+8pP6p/TJzRfNQJRdQTuvceDqPKulI8hoPavDLofg8j1cKqJPKm29AHeuHkTikumn+z1qe5JPrXzHpCEIQNCEIEkmkuSvBeEOK1ZTS2+Mwt7D+K8YV0Dwhw61DSzD9WQtPWL+pc/K+n485pDzX/Ykr2SKRXoYRxm78NoJL/EMjD9K49BWOx12NPMsjEAHYI1182VJFuYs/wDFYkRvE08y6f8AlP6sJySuglRugd0XSORSJVRLWzV9FJyVbDIT8SRruw3WMFJhs7pXSvbMvomN+tC13EKLnLHw6blcNp5L31omn0Kxzl7HmNzlU5/OoucqnOVQ3vVD3oe9Y0j1VDpFQ+TnSe9Y73qKm6TqVDpOdQe9UPkUVY6RQdJ2Kh0nOqnSIrIdLzqszc6xjJzqBkUXDK5dMTZ7VhGVLlUyNiJudWNm4la4Sq1siZGxbIrmSLXMkWQyTnUymGwZJszV7JFrmPWSx90RnsfeyvY9YMblkRv2K5RmsddXtcsKNyyGOVRkhymHKhrlY0qMr2uVjXLHaVY0oLgUTv1Kd7uDSfQotKoxWTksJqpL/FhcfQVY7Hz/AFD9eokff4ziVFpVZKYK81npr0uBU2lVAqQK5y0sui996jdFwstq6l35h3QsnDPEwSQ75J/ub+Kwqo/mDzrNphqYJT5/Ge93pA9Sk9J/UCUrpXQoJ3XT9BY9TRmN+zlJHnsNvUuXA5rr2isPIaMUDd5hDz0nM/evN5U/hh10u23CaQTXznoCEIQCEbEIEjYEJLmrz2m8PK6OyOtnE9rh229a5eV17SOHl9H6xn8onszXInCxXv8AFn8ZcNTtAqJUioletyTnYJMDqxa5jkjeO0j1rW0xvF0LbQeNQ4hF5VMSOlrge9aikP5vrXSP1Z/q4pb0ykUVFxzyUSUztUSVqGZO6A7NRulddIZl3jRubldHKB4zvA37lnOctFoTNyuiVDnsYW9hIW6eeK9kPPKD3c6pc5TcbA8ypebKsq3uWM929WyOWNI5GoVvesd71N7ljSOzUVF71jyP2qT3WWPI7NRQ+RUuk50nvVL3qS1CTpFWZRfaqnyZ5FUOlzWJlrDJM1kuWusMyc6BJmplWwbLe2avbJzrWNkKyI5edMphsmSLIjfzrXRvyWVG9ahlsGOWRG7NYMbrrJjcqks5judZDHLCjdkshjkRmsfuWQxyw2FZDHKsyy2lWAqhhurWlEXNKsBVTSptKrK5pWu0nk5LRrEX3tanf9y2DStLppLyeiVfntjt2kKwOHOPjHpSBUSc0ArzS9MLgVK6qBUg4LnLa3WQSoXQSsSqqrd+btzrY21MIom/yy49biVqqo+IOlbisBjgpI97KeO459VSf4QxE7qN07qKla4sNp2Lt1BEIcPpogLBkTR6AuK0kfK1cMflyNb2my7g0WaBlkF4vLnqHbSSuhMI3Lwu46kIQgaEWQqIpIQuaqK2ITUU8R/XYR2hcWkuHZix3jgu3OF2kcVxrFoTT4pVREW1JXDozXs8We4cdRhFIppHYvc4r6Lxpnxk5SRSM+yVpqQ/GC3OHkDEIOBeAevL1rTRAx1UkZFiCQR0LpXqWZZF7KKnvUSMroqDsiolMqJW4ZlEpXTKiVqEl1TQjFGUeiELpGueBM9ni2yzJW8OPQEZQyeheK0Sfr6J1DfkqwHtaFtA4AbuwL2V6cJj235xiF17MfzXIUDiLHfqHtWna4WUw/K9htyVymGxdWNJ2elVPmB4dqw9fLZ7e3txevl8Ue3t9/HOZkwucbg2sOtUPYTvA6/b260a+eX3qsu5z2+3t6JlUHRF21zRn7e342qdTOP64CsLyXbd/t7ewjr5/G5tv4JlVDqIk/pBboVTqB1v0o2cPb29OW943ut7dCg523O+XeoMJ+Fk/th9H29uq9TsJJ/b/YK2Jcbdqhc2KzhrMtccI2/8R9gpDCbEfn/srY3JJUCUwZYX5PDf232VIUgb+09CyXdCsFJLa7xyYOYLza/QPbvyvtjNGpbPcr4Jda4I2KqUshzDS4gfrbOxVUM75jIXG9iAOZInJhto3LKjcsGMrKjK2xLNjKyGFYkZWSw3KqMuMrJjKxGHNZMZVZZTCrmqhhVwKIubsVjdiraVYFUWNXnvCC7U0Qqzx1R6QvQtXl/CVJqaIyNv8aVgRIcZ3pgqJ2o3Lzy9MLAVJpJKlSUz6qQtYQ1rRrPe74rBxKyDNQQkiKmNRb9pM4tB6Gg/fdc5luGNdBKy2zUFQdSWn9yk5crE4uaOlp3dFljVUMlLO6GSxc3eNhG4jmWFYtRmQ0Z8FvMWI92uaNjAG9gC08TTJXU7AL3eBbrWzxB4fWyu4uP3qW/hHTGKSLpKK2ej8fLY/QxeVO30G/qXaAuR6Ew8vpVSfy9Z/Y09664Avn+VP5RD0aXRoRuTsvI6kmhCA6kIQgghCFhSO1cp0vh5HSOqG55D+0LqxXN/CBFqY0yS2UkQPYSvT404vhy1OnlEjdO4Rkdi+g4HE4slY/yXA+lYmIMMWPVQIsHSuI6Cbj0ELJcDYhRx235ZjmBymijf2tHculElQQokKwqOxBW4DioFWuCrK1CSrIUSrCoELcMvaaEu1sDxWPyXxye3YtwDlkPb2+7s0WgZ1ocVi4wB3YVu2nIZL10/WHGe1jTkPUmCbZ8OO326++sO8Ugp8o291pFl+nt9va/W78c1VygG8ZH29vYnK3I2HL29ujrgt1iTfM9agTmq+Vyztzmyi6Q3JyBt2IqROaRI23t1+3sFWXm+Xt7ersC93sVBY6wBv7e1vbcnEDmUCSeHQm1r32AG1QGtkoZnIC63lDotiVY1rzEWRuF9d2QssyHAqKGVzZXyVLmH4sWTL/4t+3cs1tF5xX2WmKxmZebhpZ6l4ZHEXuccgMyVsafR5znltRJqkbY4wHv69w6z+Pq6Gjp3wlrZGxADxomDVaek7T1lSqKQUgaAGxtPjWaNq7xozM4lwnyKxOIecdQChN2RMYSDquvrvvbich1BaGpkczWDjra23WzJ9a9XWkVDQ2M6j4xk52wDpXmaunjiu+aUFxPxhv6OKzPjX/rrXXrhp3Mmqnagad+ZNgBzrKgpBSRMtdwkz17WDujmU6yVlJHeaPVLheOmO1395/Nzb1j0M8tS+WWdxc8uA6BbZzBctm2cOm7LYMWVEseMLKjGxahmWRHkVlM2hY8YWSwKoyI9yyI9qx4wsmNVmWQ3JXNN1SxXMzRFzVaFU1WtVRY1eO8KLiNG4m+VUN+4r2LOC8P4V5LYRRx+VMT2BP5JDlBzQMig7U2i56rrzy9DOceSwWFrcvdEjnP5w02A+8rBus+BhrqAUrD+fhcXxsP7Rp+MBzgi9ucrAsQSCCCDYjeFyhs9a3Ss+uOvhuHSO+Pyb2f6Q82WPSUclW86tmRMzkld8Vg5+5SxCpZPM1sNxDC0MjB22G885Oak9iOFsMmNUoG51z1Z+pWzEmRxO0lGBs18WMl7CKF7vs29alJE593N2XWZ7ajpSi69HRaC4/X0jaiCkBZILsDnWLuhaGop5aWofBPG6OWN2q5jtoKzFonoer8G8Ifj08pF+TpzbmJcF00Ln/gyhs+vm5mNv2ldAAyXzfInOpL06cfiaEk153QIshCAHR6EI6kIIJXTQsKRXhvCPBlR1AHlMPoI9a9yvL+ECLXwFj/k5ge0EetddGcakMXj8XidGKOlrcZaysGtExpeWHevZVrMFrMKFOcObBICfzjbawNti53Tzy0lQ2eB5ZIw3BC2FXpBV1kHJPZG075GjxudfQtWZtEvPWWtBuXW2BxAPFVY0QWYdJb9jqH/AEuI+5WWAAAyCjizS7CaOQbGSSM//U96717ZlVuUSmzNgPMgqishRIVhCgVoVkKBCsKiVqGZen0Ad/zOsi+UpXjsW5a7xfxWg0EfqaTRt8uKRvoW+uAS3gvXp/q427TDm8T1I1h7H29vTFpado6c0tYXyA7VpE9ZGsoF2ez0o1uZQT1jb7kiczlkgZ3AVzYri5BIHMszaI7WIyx7knL0KwROd0ncthT0bpZTHEy+waxGzitrHhZkIjporxh3jzvOXP1XysuNtaInEOlaTLz7IHZZXXrMJw/DhTGanZLLK0C76mIhjegLNw/BsPbOXCMTubbMizR0Dvut4IwQGtFx0LMavv2mpWYjH9aeeeVzdV1TGBsNrgAdCwTqbGPLgObet5UYYwkvB37LKMeHB5ya7PbsX06eTo0j8YfJ+NqzbMyrwRjJg8PtrbnEbVh4zT1DZS+Yk0+9wO3mWwnhjoy0g2Bydbdzry2N6U8kTStLZYgcg4dy3XUzbkjpi2nbdsgVcEslm08IcCR4kcgJ681RjdVhWBUuqIm1Ne9viMc0ERZbT17FpWaTGnFQ+loKeGolyE7Bm0b7BefmkdI9z3uLnONyScyuGtq21Ix09+npRWcqppZJZHyyvc+R5u5zsyVsMHF45f8AGPuWscc1tcDF4Zf8Y+5cP67/AMbWNqyY2qtjFkxtWmZWxtushgzVTBxWQxqrOVsYWTGFSxuayGDYiLmK5oVbArmhEWNCsCg0KwBBNoXPfC0/8zh0f957vQF0NgzXNvC07/jMPZwjefSEnqVjtzghANjsUkrLzvQNhBblY5FZbcUrbDWkbJltkiY89rgSnT00EVKayrBcCbRQgkcpxJI3BS/LFYMoTFAzcyOFgA7QVzmc9NQonrKioaBNKXNGxuxo6AMljuzutlFyeKl0Too46vVJjdENUSkZ6pGy545LWuFiRvCkDYYDGXSV7wCXNp9UAc7gEM1qWojkmheGawJDmkEjftRg3i0GIyXtfUb6b+pVF7icyTbisT7mWo6dNh0g5SCKSCv5GOE3YdcfFXhdIK6PEsZnqo82uIGt5Vt61uvcW2DmQTdc6acU6amcukeDWLVwiqlP689h0Bo9ZK9kvNaARcnorC7fJLI4/SI9S9MF83WnOpL00/UIQhcmghCOpA0I7UIKkIQsKFpNMIuV0bqcs22d2FbtYONQmpwWsiG10LgOxapOLRKT043ZJSO2/HNIr67yIqVeC/R6/wAnVDsLT3KKtkHKYHXx728nIOo2/wDst17JYVObwNPMpFVUhvTgcFaVZ7SEHKBVhUCrAgVEqZFlFaRt9EJOS0qoDudIWnraV6WXxKiRth4r3D0ryWAv5LH6F/CdvpNvWvZ18ThiVS0N2SOPpXq05/FxtHtjtcbe2altKkyDWJBIBG0FZkVE0PBOtZxIyG3mVtqRCRWZYrIJZCNVt+CzocGqHtDnNDR/eW7wGkilfPFJEOWZGC0k3tvy7VmQRsEUklRFICcmAu1b84Xi1fIvE4q+l4/jaVq7ry89+THwvDXXzvew2Z8+3cVtKPBnzxB749SMm5kkcQHDmy6di2URpYCxkEPLzD9pI25vzBZAgrKhxe8udccV49Xy4j1M+3SPExOZnEK6ekpaZnJQx8sRtLhZvZ3q513OHKODiNjQbALFlbNESx12gbQhpFxqnPpSt93t7K+PWsem0onMbONdwbcbAtiZ4mghp2C+XX3LRQQudI21zs27+ZbghkTb5Od7e3avTSZmHh8jSruzLIa5guXXtz9NlTU18VPCXZRstfWO/YsCuxGKjjLpXXeM9S/39g7F4PHNI5aqRzWPvbIcAvZp0nuXztTbHqrYaRaVFwdDAbA7r5npXjJZHSvL5Dmc80nuJcXvJLjvKqc8gLvn6corgnO5yqHuTc6yrcbrGWkCVvNH23p5v8Y+5aNeh0aZelm/zB9yR2stuxqyI2qLGbFkMb6VtzSY1XsaosYr2M2IibG7FkMaoMar2tRE2hXNCrYFa0IiYU2hRCsagm0Ll3hXdrYxSN8mEntP4LqbAuTeFJ+tpHG3yYG/eUt+stV7h4jVQGgm2xNI55LzS7szGXWxF0AyZA1sbBwAAWCVsZGHFWxyQlpqw0NkiJAMlhk5t9pttHMsb3BWufqCjqC7hyLu5c4n00rpC/3bByd9cSstb/EFLEQPyhUFtrco61ulZkUX5KcZpi01YBEUTTcxnyncDzLXSjxC4uBJvcb1M+z+MzDbtwapd5UzR2A96pV1JlgI/vTuPYB3qm6n9loJt2pJoOy6Jw8hovh7LWPIgnrzW4CxMLi5HCqSK1tSFjfQFlr4t5zaZeyOghCFlQE0k0AhCEFSEXzQsKFGVnKROaf1hZSRZEcTqo+RqZYyPiuLewqlbTSKHkcerGWt+dJA6c1q7L7FZzEPLPaJV8A16atj261M49hBVKyaAa9QYh8aVj2drT61uO0aihPiOHAq8rFoidd445rKK1btIRKjvUionakCLs1Gykiy0L6B3J4hTv8AJlafSF06soDLicxEYfyhBtrAZWHeuWw+LMw8HArtzKSOanZPJNyTHta7xLlzzbhsAW92KSzFZtbENLFAQwGMNkaLEsLD4x9f4hbemwd7I2yTubGCCDygJdnwF8t5CyopYoIwykgDM7F1wXHpPG/BMNe8h7ze4uSTmV5b6r208We7CMx09m0kdsrF5HjG6pqIy14Mz8/SVmA2YeQDXOGy59uZWxR0xLRJA6aYN1nOOxp614PK8qNKsTjOXs0610v4rwmnbK8ykWYzLVtmV6KnkiYdVzmg7rleYE9RC4NgBZq7HBtxbgVXN7sqp+Uc8j0ZL5uhp6+r5HNj0mto8s/lbENpjRh90B8TwXHa0FY0QhIvLGctuSxTCQ/Wc4m4WfFAzkuUlOqwZ57/AGuvu6Glf+rN6aVIiZ6E9RBTU5laXBjd1r58F5iu0krZZhyDnstkyNmZ61nOxk1WPHD4gG08cZNhtcbjMlafEqsU1bOyKMcsXZSW+KLbl216zSO3q/5vHrZnblgV9fW4hVCjia90xIaWgZk8FjYho9ieFwcvV0j2Mcba9wQDwJBy61naNyTnSpjoHw8rd2rypyebbL8TmFvp2CPDK2r9x1mHci9j5YKh2vDUEO+KL5r3UtM1jL855OI1rRHWXPXAk2spUtBVV9Q2npoXSSu2NG1dFNBhNBVQvipYaluL1LJIY3AAMjA1iBfZ4xt6FuGQxQ4lQ1EVPDDI90kVnwCOQjVJAA2EXG1ay8+5xl0MgJGqcsjkoCB7h8UrslFT0xo4A7DWvM5casNhZYPvmHEm7bLApp6WlnwXD4KSmdT1TJhJrxtcXButbPqTJucokhfH8ZpF+Zeh0Wbejm/zPUtlpPVMxLRSirpYYW1BqZYtaNgb4o2CwWHomy9FP/mj7kjtc+m6YxXMYpNjVzI10YmSYxXsamxiuazdZEDGq1oQ1qsa1VDaLKwJNapgIJNCmAogKwBETYuQeE1+tpQW+TE1dgauM+EZ+tpdUDyWtHoWb/q3Xt5QoTUoonTSsiYLue4NA5yvNL0IBpc4BoJJ2AC5KzHsxYRnXZXBm/WZIB9ytknNOXUeHa1xflJWjx5CNvQOYKp1LXxCKUCUOkaXgtLtYW2rlMk3rE4mWG3I5KE7yYze2Qtssti5wr6SSV7bVMABLxlyrL2uecXGe+/MtZUEcn1qx21PTYt8TAqMeUXu+1b1LHyWZVgMoMPjG6na49ZJ9aw1mFAVtMzlKmJnlva3tIHrVS2OAQ+6MfoIrZOqGX6jf1JacRKx27XG3Vja3gAFJARdfFnt7AE0IUBkl0JoQCEIQUqSSAsKEdiLoG5By/TWHktI5jue1rvR+C86V6/whxFuK0826SG3Yf8AyC8gV9XRnNIeW3ZK6geGYhTuOQ5QfeqChr+Te1/kEO7M11ZYIi9z4jNAM9R7mdhssglPFmCLSOpDcgZSe3P1otnnsW7MobRxSOa97URNODUJo8Kp6kck0hppi+176xuFotKotUUUrqdsEjmOa5rYuT+KQBl1rnW+Zw+fo+dy3iu3GXnUAKSAur6IaLFduwqN9VhdC9pa0Phbdx6AuJgLs2jEjpdGqAx07pXujDQ4EeLZZ1ZtGlbb23pW26kS2L4GRMEcdnSOyAaMgpNgqmPELowyw8dxOtrcw9t6tk5WiiLCeUmffVIF9QLIjJLMoWmUnxjv6V8mtL607Z7e3U1prXd/FFPyMNS3Wc7JxBBbkfbirayI3cIhZruCQgaHGTkwMrZm6lBOwlzRYnZdd/G8OdOsxqe/bHNGpfNWPFGQ7xzn5I3qwxOfqgbSdyujgMklxa9806mripGuDbF+93BfTppTb1HTlqa8af8AsqpRFSt1prFwGTAvOY3j+o11n52sANyx8axtrA4a9yeJXkKiodUyl7zluC9la104xDwWvbVnNmbh+MSUWJmt5MSXBBaXWRi+Ktrah8kEbow/42sc+gWWtLhZVufzrlakW9y9On5GppVmtJxlMSujcHNNnDYQrpcYrKh0YqqiWoYwg6kshcOjMrBc7nVZdmtvPPtucWxubF6iFzIWU8cDAyKKK+qwcyxZqzEHSsdJPMXtPilzjcdC9DonyeGaPYnjjYWTVMLmRRBwvyd/1vSt3glcdJKSnrK+CP3TQ18IbMGAa7XH4pTLEvANqq48oxs0p183jWOfSqHVE12/nX+LkM9i6NjzGYDhWIVWGBlRPU1D46mdhH/Dgn4nXfauYudmSix7TdK9zdUuJaDe116zQ8a1BUH+b6l4++d17TQtt8On/wA31BK9lunoWM5lc1ibW2VrWrthyyTWK5rUNarGtUQNaphqYapgKoQCmBzIAUrIABTaEgFNuSCbQbLiOnz9fS+t5nAegLt42LhOmT9fSzED/NIWL/q3T9mjWZhBAxSC5tfWaDzlpA9JCw7JgkEEZEb15JelsMEdCzFoG1ERLjKAHF1g07MxbPP7ltsQhqsOoqs4hVtqxO8BkbJCQDfbzcMlppX0teeVfIKaoI/OAtJZIfKyzaTvyKg2jo2HWmrWFo/VgY4uPNcgALlMe3l1PGm+puz6FK3Uo6uoLS1j28ky+8kgnsA+5ayp+KBzrY1tX7pLWxsEcEYtHGDew49JWvmGtIxvErUPU22KkCeOMbI4Y2/ZCwllYm6+ITW3Ot2C3qWLdSOmpC9BoPDyullGSMma7+xp7159es8HUWvpC+T5OB3pIWNScUlqvbqCd1FNfIw9ZppBNA0JJqAQjNCCi6LpIWFSuldK6FB47wiQ61LRzbdV7mk8xH4LwJXS9OouU0fLj+zkab9OXrXMyvpePOaPPqdkUiARbcU0ivQ5q8YdrYlDMRYywxvJ6Wj1gpXTxkHVoZdxh1fouKiM2hdLdQykJ5WgBsrwBuDioue55u5xcec3WwwnBavF5wyAMay9nSPcLA24bT1KGJ4PWYVO6KojyFiHtzaR0rGYzhwjV0Y1ePMbmCNiYCVk1t6TC7J4PdWo0WhDj4rNZptt2lccC6r4Nq+CHAnxzSBgD3AX7V0rG6JhzvMx7epfRmoa2Fsjw1m0g2PoWVEHMeIzrEAWu7NUx4lQxXInbfapHGKBpuJ2jitxpTnpx3Ng5jTHY5ZbFhxUkbNZ7vFaduaodjtCL3nbbhcLXVmORS5NniA3AvC710Y7krq2rExVn12JsijLIjqM47yvGY1j4aSyN1zssFKvnkqLhtdSMB4yrRvwpjnl0mLUVz/MXafUYhmPc5lgSzOmfryG5VRes92F0w+NjNEP9Sg7DKLfjVIueHSJhgOfkqy9Z5oMOHxsdpexVmjwj9bHqfqas4MwwHOUNZZ5pcF349F1MS9zYEP46D0RFMLlk4HpBUYK+QRtjlhmbqywyjWY8c4WfV6aVT5KYUlPT0tPTyiZsETLNc4b3cVpxDgI/jTj0QlPU0ft/a8p6ISmGZwzqfSyugq66fVie2uDhNE9t2G/NfctE51yVnaujvzrOeiA9yV9GvnOqPRAe5MEYhg62a9zoL42GVH+d/8AULyl9GL/ANpVn1H/AIrdYLpLgGD076eGqnkD3axL4jw5grWMSW9w900BWtAXlRp1g4/av+gUfCBgzXWMkt+aIrrmPtyxL1wsrG7F48eELBQQC+b6oqY8IuBtOb5s/wCUUzH2Yl7AKYXj/hFwJvxpJvqip/CNgI2yy/VlMx9piXrwpDYvJfCJgQGc0v1ZT+EXAGtvy0v1ZT0mJetFlK68iPCPgFr8tLb/ACyn8I2AkXEstv8ALKevtcS9cDYFcE0lk5XSOvdxnd966YfCNgRaSJZfqyuT4hO2pxConabiSRzh1lctWYw3px7Y4UudRCkLW515Jl6AAXEBoJPMm5jmGz2lp4EWXt9E6WkgwuGo1mNmqXuaZXAEttsaL7CVlaS0lPNglU+YtkfDYwykDWvvbcbVwnU/LD41v+rEeRxbfXTnhUadokxSlYdjpWD7QUip4UA7HqYEX1SXdgJXWH2U612tVzO4vcfSqU5DrSOPEqKkdKd17jwZxXqq6U/qxsHaT3Lwy6N4M4tXC6yYj484aDzBo9ZK5a8/hLpp/s9tdO6iEL5j0p3QohMFTCpXTuopqYEroUUJgUXSugnrSXJUroUQmg1WlEPL6OVrRm4Rlw6RmFycnNdnq4+XpJovLYW584XGHDVJbwyXu8WfUw4aiJUSpKJXrchirQ7B6OQbY5ZGHrDSPWqIzeJp5lk1V34JK2+Uc7X9oIWJTm8LV1/8p/W0wjFThNSJm08UpuDd4zHQdytxnSGsxh5DyY4MrQtcdXr4rVoXPbGcuE+LpTq8sx+RWTshNaekBTbLIwWa4gcxUEXyVicJhb7oktm4nrUXSPP6zu1Qukelbi8piFomcMtYg7s1B8pvfWOarJUC7nWomUxBve4naqy88UnFQc7NaiZZmEi7fdLlHW25KF0rqiWseKWtzqN0KsrGB73hjGlzjsAFyVJ8csZIfE9hb8bWaRZbqOnOGaKDEIzq1NY/UDwbFjM8h02VEeLOqdHp6ComDpGysdEXnMi+YvzbVnd9NYarWS1+dbIaNYqXOApwbM1xZw8Yc3FY/wCSazkuU1G/o+ULNYa+p5Wrtsruj7TEqoIJ6l5ZBE+RwFyGi9kpIZob8rE9ljbxm2z9it1jEIwrAcPportfVAzTuGRccrDoF1jz102LYTQUVzNVRSPjDdrnA6tu7qWYtn2uGpumHLPjwGslfqxuhfZ/Juc2QEMdwKsk0cr4xOHGLlIGl7ohJd5aNpA4K7oTEtdrHijWVV0XWkW6yRcq9ZK6ot1ilrKF0XCCesUw+yrui6C3XuVIFVAqQUyLQVIFVgqYWJlqITCaQKaw1hsMMxyswnWbA5ro3/GjkbrNPOpYrj9bi2q2dzWxt2RsGq3sWtRZZxGcvPPjaU35NsZRJV+DG2JzSW/RwSHo8W3rVDldhTtVuISH5HVHW4BX+S7/ANVu2pIKFQLqugMXJaLROt+kke7pzXKhmuxaKxcjoxQM4xB3bn615vIn8MOunHvLcIuldC8GHoSumFBMFBNF1G6d1BIFCSEFCR2oQVwaAUlG6LogOYK47isXI4pVRAZNmcB2rsS5VpVFyOkVY2214d2gH1r1eLP5TDnqdNMkjemve4JEB2HVrD5DXdjh3rCpDeG3ArYU7ddlRHa5fTyWHOBf1LWUj2ta7WIGa6R7qk9srciyjysfljtRysfljtWcS1k01Hlo/LCOVj8sK4kzCSFDlo/LCOWj8sJiTKRSJUTLH5QUTKw/rBaiJQyVBxuLXQZGbnBQL28QtRCSHG+wbVUTmpkgi+sFA7ciFuGJK6W1FjxCVucdq0guldHWEW5wqPU1cgqtA6VzP3eXUfzbR6wqcKhoJtHq2rloGOlpGixLnWffitTh+KSUDJYS1k1PMLSRP2Hn5iskY7yVFLQ01LFFTTCz2FxcSbjO/VZctv8AGst1i1fJHX4IxsjoozAwP1Da4cQCPQjEMQpcM0tmmNNUSz31A0PaGG4ta1r7FocSxl2JRRMfTQRmFoYx7Na4aN21Sfj00jWvfFA6qY3VbUlp1wOPC/PZIouW20ukFTh+FVcYsx0bm24HLJR0MpojUPq3n84GuZEN19Uknp2dq01Niz4KU0kzI6qnLtYRyg+KeIIzCjJis3LwywalMIDeNkQsGneeclNs7dqZ95ei0KcA6vMmbCI9vla2SyKZ5fprimsSbQyDPhYLzrNIqqJwMLKeIB/KOa2PJ7uJTj0jrYq+auZ7nE0zdV7uSGY/FSaTmZXdDVB25F0PcJHl/itub2aLAJZeUurmaLpWHlJ2HlKg1kXSy8r0J5cfQigFMG6WXE9id2jeexBIFSBUC5rTvBHMgPaOKguCsBWOJW8CpcuBuKzMLDICmsX3UAfilSNUB+r6VnEtZZCFje677GX60/dDzsiKmJMrXK7DT/y6tPlPY37z6lhmSZ2yBx6AVnUkT4cGe57C0yT2zFtjfxSeiO1CChCBEkNNttl3DDYhBhtNENjImtHYFxWmiM9VDC0ZySNYOsgLuLQGtDRsGxeTyJ6h10v6ldO6imvG7HdO6hdSBQSTUUwVMB3QhCCm6V0IXmbF0XQhA7rnWn0HJ43HMMhLCOsgm/3hdE2LxfhDhvFRzDcXNPoK9HjzjUY1I9PDIWXheHuxTEYqNjwzlDm47gF6au0WwyCi1qKvkfPnra7MjbrX0JvETEOGHlaKdtLWxzSBzmNPjBu0i1lX7kwXhX/7aruTe+0G21JbzMItFLg18xXf7aPcuDbhX/7aqSVzP2Yhd7lwbf7v7I0e5cF3+7+xipSTM/Zhd7lwb/1/2Ee5cG/9d9hUpXVzP2mIXGnwXhXfYS9z4L5Nd2sVBUSrEz9jI5LBfIressS5PBvkqz6TFjFRK17+0ZRbgo/Y1f029yV8GH7vVH+o0epYZTjYZJWRggF7g252C5V/+ozR+Rz+61P1w/7UiMHGylqfrh3L3cOA6P0erRTQ8q9wGtKTmeNl4PF6aOjxapp4iSyN9m3222rFLxbpqYwL4P5pU/XDuS1sG81qfrh3LBJzSXXDGWfrYN5pU/XDuRr4OP3Kc5b5/wAFr0Jgy2AmwgD+zpT01B7kCpwkfwt56al3ctehMGWw91YV81H/AOS5Bq8K+aP/AMly16EwZbD3ZhfzQOuoen7swu39jt/+Q/vWuQm0y2Bq8M3YPH9fJ3pivoBswen63vPrWuTKbYMto3FKIbMGpOvWPrVsWIxyEiLBaJ1tv5q6066FoXHSUuCtq2wsmne4tfrC5GdrLnqTFIy1XMzh5N+LQtcQ7B6EEbuRsoHFYDf/AJVRD+kt9p+aWaakqY6eOGZzS14YANYDeRxXj8lqsRMZScxLZDF4Nn5JofqlL8rw/NNB9StWApK7YTMtn+WIbf2TQfUhMYywCzcNoB/QC1drphNsLltfy24bKGiH/t2qX5fn3UtGP/bN7lqRtUtqk1gy2o0gqt0VKOimZ3I/L9du5AdFOzuWrTCm2Fy2Z0gxG1hLGOiFg9Sj+XsT3VRHQxo9S1yamIGa7GcSec62bqdZQmr6mqhDKieSXVN267ibdCxEwriBfTU01XJycEbpH8GhTrsOrMOkYysp3wueNZuuLaw5lu9EKyKnE7RYVDnCxJsQ227rWdpdi7K3C4aeWobPKxwLA3PUG9Y3Tuxhcemh0Zh5bSTD2fzmu7M/UuxLlWhEfKaTwHyGvd6PxXU15/I7dNPpJNRRdebDqaajdO6IleyRcRsSugouRd3FCXSUKYAhCF5GwmkmgF5nTuIPwNslv0UzT25etelWvxzDnYrhM1GxzWPeBql2wEG66ac4vEpaMw5RS1MtHUtnhNnMPbzLbVWkpmpwyGn5KQXu/WuBfgth8HuIn97px9LuR8HmI+e0/Y7uX0N+lM5y4bbPJ7MuCS9b8HmI+eU3YUvg8xHzym+0tcun9pss8lZC9b8HmJed032u5L4PMS87pvtdyctPs2S8kUWXrfg8xLzum+13I+DzEfPKbsd3K8tPs22eRKS9afB7iI/fKb7SifB/iPndN2OVjVp9m2XkyFAhetOgGIed0/Y5R94GIed0/Y5a5KfabZeSKiV60+D+v88p+wpHwf1/nkHYVqNSn2m2zyBSzGY2r1x8H1cf3yDsKXwfVvnsHYVrkp9pss1bNKa5kLWWjc9osJC3NaiWV8sjpHuLnvN3E7yvWfB5WefQ/RKfwd1nn0P0SpF9OOlmtpeNJuUl7L4Oqvz6H6JR8HVX59D9ErXNT7Z2S8ahey+Dmr8+h+iU/g5qfP4voFXlp9myzxiS9p8HFQf4hH9AqQ8G8+/EI/qz3py0+02WeKugr2o8G8vzgz6s96l8G79+IN+rPenNT7XZZ4e6a9wPBufnEfVnvUvg3vtxH/b/ABTmp9myzwl017v4Nm/OX+1+Km3wbR78Sd1RfipzU+zZZ4MLLo8RqqBxNNM5mttG4r2rfBtT78Rl6mBTHg2o9+IVHU1vcpOtpysUs8HU1c1XLyk8he47yVSuifBtQb6+p7GdykPBth3n1V9juU5qHHZzlNdGHg2w3fW1f2P+1Sb4N8LG2rqz1t/7U56HHZzgBMBdKb4O8HG2WqP+sdysb4P8EG0VB/qlTnovHLmQUgunjQLAt8U5/rOUhoJgA/d5j/Xd3qc9F45cvTC6mNCMAH7m49Mru9Tbobo+3+HtPS93epz1OOXKU11kaJYAP4bF1k96mNFcBGzDIOw96c9TjlyNGS6+NG8Ebswyn+hdTGA4Q3ZhtMP6QU56/Rxy46MjcZEbE9a+03XZBguFjZh9N9U3uTGD4aP3Cn+qb3Jzx9Lxy8J4PWa2OyPtfUgd1XLfxXSljwUlNTOJgp4oiciWMAurgvPqW3zl0rGIwaaihYVK6LpIuoHdO6jdCB5IR2oUDQi6S8boaajdO6BE5oRvTQCE0lQIQhA0IQgEiE0iqIOVZVjlArcIrKgpuUF0hCKiVIqJW4REpIcldbEkwo3TBREkii6V0BdSUbpohoQi+aBoSTRQhK6EEgmEgmEEgmo3QCgkmo3TuoJXQop3UU0JXTuqGmooQSuhRTugkhRui6IldF1G6Lq4EkwVDWTBTAldCjrZIumBK6FFO6YDui6W9F1cCV0XUUKYEwTxQobUJgTui4QheB0Fwi6EIC4UghCAui6EIApgiyEKguEXQhFK4USUIVhEXFVkoQtwiBIUboQukJKJKiXBCF0hECUroQtILqQKEIDWyUdZCFQwVIFCFEO6MkIQF7IuhCKV07oQqh3TuhCKd0XQhA9ZAchCgesnrIQgNZPWyQhAtZPWQhAayLoQiwNZF0IVQayLoQgd0AoQgesjWQhA7ov2oQgLhGshCAJRdCECuhCEH//Z</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>box02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>New box</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
         <v>2026-08-03</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -482,79 +462,9 @@
         <v>Notes</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>box01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>IEC power cable</v>
-      </c>
-      <c r="C2" t="str">
-        <v>5</v>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>box01</v>
-      </c>
-      <c r="B3" t="str">
-        <v>HDMI cables</v>
-      </c>
-      <c r="C3" t="str">
-        <v>6</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>box01</v>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>box02</v>
-      </c>
-      <c r="B5" t="str">
-        <v xml:space="preserve">1060ti </v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>box02</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2060ti</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory — 5/8/2026, 8:35:19 am
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,16 +437,33 @@
         <v>2026-08-03</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>B002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>New box</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-08-04</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -462,9 +479,23 @@
         <v>Notes</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>B002</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Hko</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>H</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory — 8/8/2026, 8:50:08 am
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -463,7 +463,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -493,9 +493,107 @@
         <v>H</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Ktm mufler</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B4" t="str">
+        <v xml:space="preserve">Ktm radiator </v>
+      </c>
+      <c r="C4" t="str">
+        <v>2</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Chain</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Rear shock</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Ktm cdi</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B8" t="str">
+        <v xml:space="preserve">Camp shower </v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>B001</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory — 8/8/2026, 11:23:16 AM
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -425,7 +425,7 @@
         <v>B001</v>
       </c>
       <c r="B2" t="str">
-        <v>New box</v>
+        <v>Motorbike parts</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -454,16 +454,50 @@
         <v>2026-08-04</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>B003</v>
+      </c>
+      <c r="B4" t="str">
+        <v xml:space="preserve">decorations </v>
+      </c>
+      <c r="C4" t="str">
+        <v>storeroom top shelf</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-08-07</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>box electrical</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-08-08</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -591,9 +625,149 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B10" t="str">
+        <v xml:space="preserve">ps4 pro </v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="str">
+        <v>needs 3.3v reg</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B11" t="str">
+        <v>rc control</v>
+      </c>
+      <c r="C11" t="str">
+        <v>2</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B12" t="str">
+        <v>celfi go</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B13" t="str">
+        <v>catch can</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B14" t="str">
+        <v>ctech batty charger</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B15" t="str">
+        <v>dell charger</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B16" t="str">
+        <v>dremill bits</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B17" t="str">
+        <v>nissan shunt</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory — 8/8/2026, 1:46:46 PM
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -497,7 +497,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -742,7 +742,7 @@
         <v>B004</v>
       </c>
       <c r="B18" t="str">
-        <v/>
+        <v>heat shrink</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -756,18 +756,46 @@
         <v>B004</v>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>2 core cable roll</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
       <c r="D19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B20" t="str">
+        <v>36v lith bms</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>B004</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>